<commit_message>
KPI actualizado 2026-07-03 15:19 UTC
</commit_message>
<xml_diff>
--- a/data/50001525 - ZITRON PERU METRO LIMA E07.xlsx
+++ b/data/50001525 - ZITRON PERU METRO LIMA E07.xlsx
@@ -3417,7 +3417,7 @@
       </c>
       <c r="C28" s="6"/>
       <c r="D28" s="5">
-        <v>46193.195807870376</v>
+        <v>46206.57726722222</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>105</v>
@@ -3545,7 +3545,7 @@
       </c>
       <c r="C30" s="6"/>
       <c r="D30" s="5">
-        <v>46193.19580785879</v>
+        <v>46206.577005486106</v>
       </c>
       <c r="E30" s="6" t="s">
         <v>114</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-07-06 11:36 UTC
</commit_message>
<xml_diff>
--- a/data/50001525 - ZITRON PERU METRO LIMA E07.xlsx
+++ b/data/50001525 - ZITRON PERU METRO LIMA E07.xlsx
@@ -6186,7 +6186,7 @@
       </c>
       <c r="C75" s="9"/>
       <c r="D75" s="8">
-        <v>46114.63343645833</v>
+        <v>46209.20762703704</v>
       </c>
       <c r="E75" s="9" t="s">
         <v>261</v>
@@ -6233,8 +6233,8 @@
       <c r="S75" s="9">
         <v>0</v>
       </c>
-      <c r="T75" s="11" t="s">
-        <v>53</v>
+      <c r="T75" s="12" t="s">
+        <v>167</v>
       </c>
       <c r="U75" s="10" t="s">
         <v>54</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-07-06 14:35 UTC
</commit_message>
<xml_diff>
--- a/data/50001525 - ZITRON PERU METRO LIMA E07.xlsx
+++ b/data/50001525 - ZITRON PERU METRO LIMA E07.xlsx
@@ -3110,7 +3110,7 @@
       </c>
       <c r="C23" s="9"/>
       <c r="D23" s="8">
-        <v>46205.72132123842</v>
+        <v>46209.59541466435</v>
       </c>
       <c r="E23" s="9" t="s">
         <v>88</v>
@@ -3287,9 +3287,11 @@
       <c r="B26" s="5">
         <v>46108.75688076389</v>
       </c>
-      <c r="C26" s="6"/>
+      <c r="C26" s="5">
+        <v>46209.595404629625</v>
+      </c>
       <c r="D26" s="5">
-        <v>46205.72131620371</v>
+        <v>46209.59540697916</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>98</v>
@@ -3417,7 +3419,7 @@
       </c>
       <c r="C28" s="6"/>
       <c r="D28" s="5">
-        <v>46206.57726722222</v>
+        <v>46209.59805664352</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>105</v>
@@ -3462,13 +3464,13 @@
         <v>46192</v>
       </c>
       <c r="S28" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T28" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="U28" s="12" t="s">
-        <v>90</v>
+      <c r="U28" s="11" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.25">
@@ -4161,7 +4163,7 @@
       </c>
       <c r="C40" s="6"/>
       <c r="D40" s="5">
-        <v>46205.7213208912</v>
+        <v>46209.595412939816</v>
       </c>
       <c r="E40" s="6" t="s">
         <v>145</v>
@@ -4604,7 +4606,7 @@
       </c>
       <c r="C47" s="9"/>
       <c r="D47" s="8">
-        <v>46199.16861097222</v>
+        <v>46209.598061192126</v>
       </c>
       <c r="E47" s="9" t="s">
         <v>109</v>

</xml_diff>

<commit_message>
Actualiza portafolio 2026-07-08 20:35 UTC
</commit_message>
<xml_diff>
--- a/data/50001525 - ZITRON PERU METRO LIMA E07.xlsx
+++ b/data/50001525 - ZITRON PERU METRO LIMA E07.xlsx
@@ -4289,7 +4289,7 @@
       </c>
       <c r="C42" s="6"/>
       <c r="D42" s="5">
-        <v>46182.693445439814</v>
+        <v>46211.84653167824</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>151</v>
@@ -4478,9 +4478,11 @@
       <c r="B45" s="8">
         <v>46108.7570218287</v>
       </c>
-      <c r="C45" s="9"/>
+      <c r="C45" s="8">
+        <v>46211.84652571759</v>
+      </c>
       <c r="D45" s="8">
-        <v>46199.811805694444</v>
+        <v>46211.84652803241</v>
       </c>
       <c r="E45" s="9" t="s">
         <v>160</v>
@@ -5257,7 +5259,7 @@
       </c>
       <c r="C58" s="6"/>
       <c r="D58" s="5">
-        <v>46141.52778395833</v>
+        <v>46211.84618952546</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>202</v>
@@ -5302,9 +5304,11 @@
       <c r="B59" s="8">
         <v>46108.75712325232</v>
       </c>
-      <c r="C59" s="9"/>
+      <c r="C59" s="8">
+        <v>46211.846184131944</v>
+      </c>
       <c r="D59" s="8">
-        <v>46210.49827609953</v>
+        <v>46211.84618561342</v>
       </c>
       <c r="E59" s="9" t="s">
         <v>205</v>
@@ -5347,13 +5351,13 @@
         <v>46127</v>
       </c>
       <c r="S59" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T59" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="U59" s="12" t="s">
-        <v>90</v>
+      <c r="U59" s="11" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="60" spans="1:21" x14ac:dyDescent="0.25">
@@ -5363,9 +5367,11 @@
       <c r="B60" s="5">
         <v>46114.552579166666</v>
       </c>
-      <c r="C60" s="6"/>
+      <c r="C60" s="5">
+        <v>46211.84604746528</v>
+      </c>
       <c r="D60" s="5">
-        <v>46127.171562662035</v>
+        <v>46211.84604957176</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>211</v>
@@ -5416,9 +5422,11 @@
       <c r="B61" s="8">
         <v>46114.552773240735</v>
       </c>
-      <c r="C61" s="9"/>
+      <c r="C61" s="8">
+        <v>46211.84605395833</v>
+      </c>
       <c r="D61" s="8">
-        <v>46127.17156420139</v>
+        <v>46211.846055462964</v>
       </c>
       <c r="E61" s="9" t="s">
         <v>216</v>
@@ -5534,7 +5542,7 @@
       </c>
       <c r="C63" s="9"/>
       <c r="D63" s="8">
-        <v>46189.16802</v>
+        <v>46211.846533206015</v>
       </c>
       <c r="E63" s="9" t="s">
         <v>211</v>
@@ -5587,7 +5595,7 @@
       </c>
       <c r="C64" s="6"/>
       <c r="D64" s="5">
-        <v>46189.16802199074</v>
+        <v>46211.84653444444</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>216</v>
@@ -5640,7 +5648,7 @@
       </c>
       <c r="C65" s="9"/>
       <c r="D65" s="8">
-        <v>46191.171331157406</v>
+        <v>46211.84618984954</v>
       </c>
       <c r="E65" s="9" t="s">
         <v>108</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-08-13 14:30 UTC
</commit_message>
<xml_diff>
--- a/data/50001525 - ZITRON PERU METRO LIMA E07.xlsx
+++ b/data/50001525 - ZITRON PERU METRO LIMA E07.xlsx
@@ -2434,7 +2434,7 @@
       </c>
       <c r="C12" s="6"/>
       <c r="D12" s="5">
-        <v>46240.18483663195</v>
+        <v>46247.16736709491</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>51</v>
@@ -2497,7 +2497,7 @@
       </c>
       <c r="C13" s="9"/>
       <c r="D13" s="8">
-        <v>46111.57933724537</v>
+        <v>46247.16738287037</v>
       </c>
       <c r="E13" s="9" t="s">
         <v>56</v>
@@ -2550,7 +2550,7 @@
       </c>
       <c r="C14" s="6"/>
       <c r="D14" s="5">
-        <v>46111.57933446759</v>
+        <v>46247.16738408565</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>60</v>
@@ -2603,7 +2603,7 @@
       </c>
       <c r="C15" s="9"/>
       <c r="D15" s="8">
-        <v>46111.579331643516</v>
+        <v>46247.1673853588</v>
       </c>
       <c r="E15" s="9" t="s">
         <v>63</v>
@@ -2656,7 +2656,7 @@
       </c>
       <c r="C16" s="6"/>
       <c r="D16" s="5">
-        <v>46111.579327326384</v>
+        <v>46247.167386597226</v>
       </c>
       <c r="E16" s="6" t="s">
         <v>66</v>
@@ -6242,7 +6242,7 @@
       </c>
       <c r="C76" s="6"/>
       <c r="D76" s="5">
-        <v>46221.31555423611</v>
+        <v>46246.95004469907</v>
       </c>
       <c r="E76" s="6" t="s">
         <v>263</v>
@@ -6287,9 +6287,11 @@
       <c r="B77" s="8">
         <v>46111.505495046295</v>
       </c>
-      <c r="C77" s="9"/>
+      <c r="C77" s="8">
+        <v>46246.950038807874</v>
+      </c>
       <c r="D77" s="8">
-        <v>46226.19708370371</v>
+        <v>46246.95005820601</v>
       </c>
       <c r="E77" s="9" t="s">
         <v>266</v>
@@ -6334,13 +6336,13 @@
         <v>46225</v>
       </c>
       <c r="S77" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T77" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="U77" s="10" t="s">
-        <v>54</v>
+      <c r="U77" s="11" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="78" spans="1:21" x14ac:dyDescent="0.25">
@@ -6352,7 +6354,7 @@
       </c>
       <c r="C78" s="6"/>
       <c r="D78" s="5">
-        <v>46246.19524059028</v>
+        <v>46246.95045744213</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>271</v>
@@ -6402,8 +6404,8 @@
       <c r="T78" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="U78" s="10" t="s">
-        <v>54</v>
+      <c r="U78" s="12" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="79" spans="1:21" x14ac:dyDescent="0.25">
@@ -6415,7 +6417,7 @@
       </c>
       <c r="C79" s="9"/>
       <c r="D79" s="8">
-        <v>46245.167413460644</v>
+        <v>46246.95004574074</v>
       </c>
       <c r="E79" s="9" t="s">
         <v>211</v>
@@ -6468,7 +6470,7 @@
       </c>
       <c r="C80" s="6"/>
       <c r="D80" s="5">
-        <v>46245.167414490745</v>
+        <v>46246.95004674769</v>
       </c>
       <c r="E80" s="6" t="s">
         <v>216</v>
@@ -6521,7 +6523,7 @@
       </c>
       <c r="C81" s="9"/>
       <c r="D81" s="8">
-        <v>46240.18483673611</v>
+        <v>46247.1673787037</v>
       </c>
       <c r="E81" s="9" t="s">
         <v>278</v>
@@ -6584,7 +6586,7 @@
       </c>
       <c r="C82" s="6"/>
       <c r="D82" s="5">
-        <v>46227.7225096412</v>
+        <v>46247.16738049769</v>
       </c>
       <c r="E82" s="6" t="s">
         <v>211</v>
@@ -6637,7 +6639,7 @@
       </c>
       <c r="C83" s="9"/>
       <c r="D83" s="8">
-        <v>46227.722510057865</v>
+        <v>46247.167381701394</v>
       </c>
       <c r="E83" s="9" t="s">
         <v>216</v>
@@ -6863,7 +6865,7 @@
       </c>
       <c r="C87" s="9"/>
       <c r="D87" s="8">
-        <v>46240.18483702546</v>
+        <v>46247.1673696875</v>
       </c>
       <c r="E87" s="9" t="s">
         <v>294</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-08-21 13:54 UTC
</commit_message>
<xml_diff>
--- a/data/50001525 - ZITRON PERU METRO LIMA E07.xlsx
+++ b/data/50001525 - ZITRON PERU METRO LIMA E07.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1758" uniqueCount="438">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1758" uniqueCount="439">
   <si>
     <t>50001525- ZITRON PERU METRO DE LIMA  ESTACION 07</t>
   </si>
@@ -824,6 +824,9 @@
   </si>
   <si>
     <t>Armado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Caldereria,Control de calidad Armado </t>
   </si>
   <si>
     <t>1213869987281817</t>
@@ -6351,7 +6354,7 @@
       </c>
       <c r="C78" s="6"/>
       <c r="D78" s="5">
-        <v>46247.95303712963</v>
+        <v>46255.55279185185</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>270</v>
@@ -6387,7 +6390,7 @@
         <v>219</v>
       </c>
       <c r="P78" s="6" t="s">
-        <v>262</v>
+        <v>271</v>
       </c>
       <c r="Q78" s="5">
         <v>46226</v>
@@ -6407,7 +6410,7 @@
     </row>
     <row r="79" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A79" s="7" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B79" s="8">
         <v>46111.52633317129</v>
@@ -6447,10 +6450,10 @@
         <v>270</v>
       </c>
       <c r="O79" s="9" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="P79" s="9" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="Q79" s="9"/>
       <c r="R79" s="9"/>
@@ -6460,7 +6463,7 @@
     </row>
     <row r="80" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A80" s="4" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B80" s="5">
         <v>46111.526644375</v>
@@ -6500,10 +6503,10 @@
         <v>270</v>
       </c>
       <c r="O80" s="6" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="P80" s="6" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="Q80" s="6"/>
       <c r="R80" s="6"/>
@@ -6513,7 +6516,7 @@
     </row>
     <row r="81" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A81" s="7" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B81" s="8">
         <v>46111.50563458333</v>
@@ -6523,7 +6526,7 @@
         <v>46248.169711875</v>
       </c>
       <c r="E81" s="9" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="F81" s="9" t="s">
         <v>26</v>
@@ -6576,7 +6579,7 @@
     </row>
     <row r="82" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A82" s="4" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B82" s="5">
         <v>46111.526916469906</v>
@@ -6613,13 +6616,13 @@
         <v>26</v>
       </c>
       <c r="N82" s="6" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="O82" s="6" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="P82" s="6" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="Q82" s="6"/>
       <c r="R82" s="6"/>
@@ -6629,7 +6632,7 @@
     </row>
     <row r="83" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A83" s="7" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B83" s="8">
         <v>46111.52699828704</v>
@@ -6666,13 +6669,13 @@
         <v>26</v>
       </c>
       <c r="N83" s="9" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="O83" s="9" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="P83" s="9" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="Q83" s="9"/>
       <c r="R83" s="9"/>
@@ -6682,7 +6685,7 @@
     </row>
     <row r="84" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A84" s="4" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B84" s="5">
         <v>46108.75714884259</v>
@@ -6692,7 +6695,7 @@
         <v>46221.1155655787</v>
       </c>
       <c r="E84" s="6" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="F84" s="6" t="s">
         <v>25</v>
@@ -6716,7 +6719,7 @@
         <v>26</v>
       </c>
       <c r="O84" s="6" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="P84" s="6" t="s">
         <v>26</v>
@@ -6729,7 +6732,7 @@
     </row>
     <row r="85" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A85" s="7" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B85" s="8">
         <v>46108.75715243055</v>
@@ -6739,7 +6742,7 @@
         <v>46185.184959907405</v>
       </c>
       <c r="E85" s="9" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="F85" s="9" t="s">
         <v>26</v>
@@ -6766,13 +6769,13 @@
         <v>26</v>
       </c>
       <c r="N85" s="9" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="O85" s="9" t="s">
         <v>147</v>
       </c>
       <c r="P85" s="9" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="Q85" s="8">
         <v>46183</v>
@@ -6792,7 +6795,7 @@
     </row>
     <row r="86" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A86" s="4" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B86" s="5">
         <v>46108.75715773148</v>
@@ -6829,13 +6832,13 @@
         <v>26</v>
       </c>
       <c r="N86" s="6" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="O86" s="6" t="s">
         <v>138</v>
       </c>
       <c r="P86" s="6" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="Q86" s="5">
         <v>46239</v>
@@ -6855,7 +6858,7 @@
     </row>
     <row r="87" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A87" s="7" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="B87" s="8">
         <v>46108.75716349537</v>
@@ -6865,7 +6868,7 @@
         <v>46248.16971915509</v>
       </c>
       <c r="E87" s="9" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="F87" s="9" t="s">
         <v>26</v>
@@ -6892,13 +6895,13 @@
         <v>26</v>
       </c>
       <c r="N87" s="9" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="O87" s="9" t="s">
         <v>129</v>
       </c>
       <c r="P87" s="9" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="Q87" s="8">
         <v>46246</v>
@@ -6918,7 +6921,7 @@
     </row>
     <row r="88" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A88" s="4" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B88" s="5">
         <v>46108.75716875</v>
@@ -6928,7 +6931,7 @@
         <v>46111.59782981481</v>
       </c>
       <c r="E88" s="6" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="F88" s="6" t="s">
         <v>26</v>
@@ -6955,13 +6958,13 @@
         <v>26</v>
       </c>
       <c r="N88" s="6" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="O88" s="6" t="s">
         <v>156</v>
       </c>
       <c r="P88" s="6" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="Q88" s="5">
         <v>46273</v>
@@ -6981,7 +6984,7 @@
     </row>
     <row r="89" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A89" s="7" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B89" s="8">
         <v>46108.75717430556</v>
@@ -6991,7 +6994,7 @@
         <v>46224.18129432871</v>
       </c>
       <c r="E89" s="9" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="F89" s="9" t="s">
         <v>26</v>
@@ -7018,7 +7021,7 @@
         <v>26</v>
       </c>
       <c r="N89" s="9" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="O89" s="9" t="s">
         <v>178</v>
@@ -7044,7 +7047,7 @@
     </row>
     <row r="90" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A90" s="4" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B90" s="5">
         <v>46108.75717877314</v>
@@ -7054,7 +7057,7 @@
         <v>46240.16751195602</v>
       </c>
       <c r="E90" s="6" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="F90" s="6" t="s">
         <v>26</v>
@@ -7079,13 +7082,13 @@
         <v>26</v>
       </c>
       <c r="N90" s="6" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="O90" s="6" t="s">
         <v>245</v>
       </c>
       <c r="P90" s="6" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="Q90" s="5">
         <v>46231</v>
@@ -7105,7 +7108,7 @@
     </row>
     <row r="91" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A91" s="7" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B91" s="8">
         <v>46108.822037094906</v>
@@ -7115,7 +7118,7 @@
         <v>46185.18495945602</v>
       </c>
       <c r="E91" s="9" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="F91" s="9" t="s">
         <v>26</v>
@@ -7142,13 +7145,13 @@
         <v>26</v>
       </c>
       <c r="N91" s="9" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="O91" s="9" t="s">
         <v>198</v>
       </c>
       <c r="P91" s="9" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="Q91" s="8">
         <v>46183</v>
@@ -7168,7 +7171,7 @@
     </row>
     <row r="92" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A92" s="4" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B92" s="5">
         <v>46108.757183124995</v>
@@ -7178,7 +7181,7 @@
         <v>46221.36615074074</v>
       </c>
       <c r="E92" s="6" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="F92" s="6" t="s">
         <v>25</v>
@@ -7202,7 +7205,7 @@
         <v>26</v>
       </c>
       <c r="O92" s="6" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="P92" s="6" t="s">
         <v>26</v>
@@ -7215,7 +7218,7 @@
     </row>
     <row r="93" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A93" s="7" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="B93" s="8">
         <v>46108.757186296294</v>
@@ -7225,7 +7228,7 @@
         <v>46223.59523664352</v>
       </c>
       <c r="E93" s="9" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="F93" s="9" t="s">
         <v>26</v>
@@ -7252,13 +7255,13 @@
         <v>26</v>
       </c>
       <c r="N93" s="9" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="O93" s="9" t="s">
         <v>219</v>
       </c>
       <c r="P93" s="9" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="Q93" s="8">
         <v>46248</v>
@@ -7278,7 +7281,7 @@
     </row>
     <row r="94" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A94" s="4" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B94" s="5">
         <v>46111.52720202546</v>
@@ -7315,13 +7318,13 @@
         <v>26</v>
       </c>
       <c r="N94" s="6" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="O94" s="6" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="P94" s="6" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="Q94" s="6"/>
       <c r="R94" s="6"/>
@@ -7331,7 +7334,7 @@
     </row>
     <row r="95" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A95" s="7" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B95" s="8">
         <v>46111.52733795139</v>
@@ -7368,13 +7371,13 @@
         <v>26</v>
       </c>
       <c r="N95" s="9" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="O95" s="9" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="P95" s="9" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="Q95" s="9"/>
       <c r="R95" s="9"/>
@@ -7384,7 +7387,7 @@
     </row>
     <row r="96" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A96" s="4" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="B96" s="5">
         <v>46108.75720997685</v>
@@ -7394,7 +7397,7 @@
         <v>46223.595235995366</v>
       </c>
       <c r="E96" s="6" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="F96" s="6" t="s">
         <v>26</v>
@@ -7421,13 +7424,13 @@
         <v>26</v>
       </c>
       <c r="N96" s="6" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="O96" s="6" t="s">
         <v>219</v>
       </c>
       <c r="P96" s="6" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="Q96" s="5">
         <v>46268</v>
@@ -7447,7 +7450,7 @@
     </row>
     <row r="97" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A97" s="7" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="B97" s="8">
         <v>46111.52790079861</v>
@@ -7484,13 +7487,13 @@
         <v>26</v>
       </c>
       <c r="N97" s="9" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="O97" s="9" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="P97" s="9" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="Q97" s="9"/>
       <c r="R97" s="9"/>
@@ -7500,7 +7503,7 @@
     </row>
     <row r="98" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A98" s="4" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="B98" s="5">
         <v>46111.52796104166</v>
@@ -7537,13 +7540,13 @@
         <v>26</v>
       </c>
       <c r="N98" s="6" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="O98" s="6" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="P98" s="6" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="Q98" s="6"/>
       <c r="R98" s="6"/>
@@ -7553,7 +7556,7 @@
     </row>
     <row r="99" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A99" s="7" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="B99" s="8">
         <v>46108.75719767361</v>
@@ -7563,7 +7566,7 @@
         <v>46223.5952353125</v>
       </c>
       <c r="E99" s="9" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="F99" s="9" t="s">
         <v>26</v>
@@ -7590,13 +7593,13 @@
         <v>26</v>
       </c>
       <c r="N99" s="9" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="O99" s="9" t="s">
         <v>219</v>
       </c>
       <c r="P99" s="9" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="Q99" s="8">
         <v>46272</v>
@@ -7616,7 +7619,7 @@
     </row>
     <row r="100" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A100" s="4" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="B100" s="5">
         <v>46111.52756633102</v>
@@ -7653,13 +7656,13 @@
         <v>26</v>
       </c>
       <c r="N100" s="6" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="O100" s="6" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="P100" s="6" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="Q100" s="6"/>
       <c r="R100" s="6"/>
@@ -7669,7 +7672,7 @@
     </row>
     <row r="101" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A101" s="7" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="B101" s="8">
         <v>46111.527622395835</v>
@@ -7706,13 +7709,13 @@
         <v>26</v>
       </c>
       <c r="N101" s="9" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="O101" s="9" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="P101" s="9" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="Q101" s="9"/>
       <c r="R101" s="9"/>
@@ -7722,7 +7725,7 @@
     </row>
     <row r="102" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A102" s="4" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="B102" s="5">
         <v>46108.75720341435</v>
@@ -7732,7 +7735,7 @@
         <v>46223.595234629625</v>
       </c>
       <c r="E102" s="6" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="F102" s="6" t="s">
         <v>26</v>
@@ -7759,13 +7762,13 @@
         <v>26</v>
       </c>
       <c r="N102" s="6" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="O102" s="6" t="s">
         <v>219</v>
       </c>
       <c r="P102" s="6" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="Q102" s="5">
         <v>46274</v>
@@ -7785,7 +7788,7 @@
     </row>
     <row r="103" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A103" s="7" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="B103" s="8">
         <v>46111.52775804398</v>
@@ -7822,13 +7825,13 @@
         <v>26</v>
       </c>
       <c r="N103" s="9" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="O103" s="9" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="P103" s="9" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="Q103" s="9"/>
       <c r="R103" s="9"/>
@@ -7838,7 +7841,7 @@
     </row>
     <row r="104" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A104" s="4" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="B104" s="5">
         <v>46111.52780829861</v>
@@ -7875,13 +7878,13 @@
         <v>26</v>
       </c>
       <c r="N104" s="6" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="O104" s="6" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="P104" s="6" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="Q104" s="6"/>
       <c r="R104" s="6"/>
@@ -7891,7 +7894,7 @@
     </row>
     <row r="105" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A105" s="7" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="B105" s="8">
         <v>46108.757191412034</v>
@@ -7901,7 +7904,7 @@
         <v>46223.59523400463</v>
       </c>
       <c r="E105" s="9" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="F105" s="9" t="s">
         <v>26</v>
@@ -7928,13 +7931,13 @@
         <v>26</v>
       </c>
       <c r="N105" s="9" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="O105" s="9" t="s">
         <v>219</v>
       </c>
       <c r="P105" s="9" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="Q105" s="8">
         <v>46276</v>
@@ -7954,7 +7957,7 @@
     </row>
     <row r="106" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A106" s="4" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="B106" s="5">
         <v>46111.527446493055</v>
@@ -7991,13 +7994,13 @@
         <v>26</v>
       </c>
       <c r="N106" s="6" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="O106" s="6" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="P106" s="6" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="Q106" s="6"/>
       <c r="R106" s="6"/>
@@ -8007,7 +8010,7 @@
     </row>
     <row r="107" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A107" s="7" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="B107" s="8">
         <v>46111.52746010417</v>
@@ -8044,13 +8047,13 @@
         <v>26</v>
       </c>
       <c r="N107" s="9" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="O107" s="9" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="P107" s="9" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="Q107" s="9"/>
       <c r="R107" s="9"/>
@@ -8060,7 +8063,7 @@
     </row>
     <row r="108" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A108" s="4" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B108" s="5">
         <v>46108.757217025464</v>
@@ -8070,7 +8073,7 @@
         <v>46245.73985467592</v>
       </c>
       <c r="E108" s="6" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="F108" s="6" t="s">
         <v>26</v>
@@ -8097,13 +8100,13 @@
         <v>26</v>
       </c>
       <c r="N108" s="6" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="O108" s="6" t="s">
         <v>219</v>
       </c>
       <c r="P108" s="6" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="Q108" s="5">
         <v>46280</v>
@@ -8123,7 +8126,7 @@
     </row>
     <row r="109" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A109" s="7" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="B109" s="8">
         <v>46111.528031932874</v>
@@ -8158,13 +8161,13 @@
         <v>26</v>
       </c>
       <c r="N109" s="9" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="O109" s="9" t="s">
         <v>210</v>
       </c>
       <c r="P109" s="9" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="Q109" s="9"/>
       <c r="R109" s="9"/>
@@ -8174,7 +8177,7 @@
     </row>
     <row r="110" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A110" s="4" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="B110" s="5">
         <v>46111.52811128472</v>
@@ -8209,13 +8212,13 @@
         <v>26</v>
       </c>
       <c r="N110" s="6" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="O110" s="6" t="s">
         <v>215</v>
       </c>
       <c r="P110" s="6" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="Q110" s="6"/>
       <c r="R110" s="6"/>
@@ -8225,7 +8228,7 @@
     </row>
     <row r="111" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A111" s="7" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B111" s="8">
         <v>46108.75727585648</v>
@@ -8235,7 +8238,7 @@
         <v>46223.595232754626</v>
       </c>
       <c r="E111" s="9" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="F111" s="9" t="s">
         <v>26</v>
@@ -8260,13 +8263,13 @@
         <v>26</v>
       </c>
       <c r="N111" s="9" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="O111" s="9" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="P111" s="9" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="Q111" s="8">
         <v>46286</v>
@@ -8286,7 +8289,7 @@
     </row>
     <row r="112" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A112" s="4" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="B112" s="5">
         <v>46111.5281812037</v>
@@ -8321,13 +8324,13 @@
         <v>26</v>
       </c>
       <c r="N112" s="6" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="O112" s="6" t="s">
         <v>210</v>
       </c>
       <c r="P112" s="6" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="Q112" s="6"/>
       <c r="R112" s="6"/>
@@ -8337,7 +8340,7 @@
     </row>
     <row r="113" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A113" s="7" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="B113" s="8">
         <v>46111.528266423615</v>
@@ -8372,13 +8375,13 @@
         <v>26</v>
       </c>
       <c r="N113" s="9" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="O113" s="9" t="s">
         <v>241</v>
       </c>
       <c r="P113" s="9" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="Q113" s="9"/>
       <c r="R113" s="9"/>
@@ -8388,7 +8391,7 @@
     </row>
     <row r="114" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A114" s="4" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="B114" s="5">
         <v>46108.757283217594</v>
@@ -8398,7 +8401,7 @@
         <v>46221.10727317129</v>
       </c>
       <c r="E114" s="6" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="F114" s="6" t="s">
         <v>25</v>
@@ -8422,7 +8425,7 @@
         <v>26</v>
       </c>
       <c r="O114" s="6" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="P114" s="6" t="s">
         <v>26</v>
@@ -8435,7 +8438,7 @@
     </row>
     <row r="115" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A115" s="7" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="B115" s="8">
         <v>46108.757287430555</v>
@@ -8445,16 +8448,16 @@
         <v>46114.63723893519</v>
       </c>
       <c r="E115" s="9" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="F115" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G115" s="9" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="H115" s="9" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="I115" s="8">
         <v>46287</v>
@@ -8472,13 +8475,13 @@
         <v>26</v>
       </c>
       <c r="N115" s="9" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="O115" s="9" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="P115" s="9" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="Q115" s="8">
         <v>46287</v>
@@ -8498,7 +8501,7 @@
     </row>
     <row r="116" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A116" s="4" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="B116" s="5">
         <v>46111.52846596065</v>
@@ -8514,10 +8517,10 @@
         <v>26</v>
       </c>
       <c r="G116" s="6" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="H116" s="6" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="I116" s="6"/>
       <c r="J116" s="5">
@@ -8533,13 +8536,13 @@
         <v>26</v>
       </c>
       <c r="N116" s="6" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="O116" s="6" t="s">
         <v>210</v>
       </c>
       <c r="P116" s="6" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="Q116" s="6"/>
       <c r="R116" s="6"/>
@@ -8549,7 +8552,7 @@
     </row>
     <row r="117" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A117" s="7" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="B117" s="8">
         <v>46111.528518067134</v>
@@ -8565,10 +8568,10 @@
         <v>26</v>
       </c>
       <c r="G117" s="9" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="H117" s="9" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="I117" s="9"/>
       <c r="J117" s="8">
@@ -8584,13 +8587,13 @@
         <v>26</v>
       </c>
       <c r="N117" s="9" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="O117" s="9" t="s">
         <v>215</v>
       </c>
       <c r="P117" s="9" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="Q117" s="9"/>
       <c r="R117" s="9"/>
@@ -8600,7 +8603,7 @@
     </row>
     <row r="118" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A118" s="4" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="B118" s="5">
         <v>46111.531216006944</v>
@@ -8616,10 +8619,10 @@
         <v>26</v>
       </c>
       <c r="G118" s="6" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="H118" s="6" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="I118" s="6"/>
       <c r="J118" s="5">
@@ -8635,13 +8638,13 @@
         <v>26</v>
       </c>
       <c r="N118" s="6" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="O118" s="6" t="s">
         <v>55</v>
       </c>
       <c r="P118" s="6" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="Q118" s="6"/>
       <c r="R118" s="6"/>
@@ -8651,7 +8654,7 @@
     </row>
     <row r="119" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A119" s="7" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="B119" s="8">
         <v>46111.53129275463</v>
@@ -8667,10 +8670,10 @@
         <v>26</v>
       </c>
       <c r="G119" s="9" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="H119" s="9" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="I119" s="9"/>
       <c r="J119" s="8">
@@ -8686,13 +8689,13 @@
         <v>26</v>
       </c>
       <c r="N119" s="9" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="O119" s="9" t="s">
         <v>59</v>
       </c>
       <c r="P119" s="9" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="Q119" s="9"/>
       <c r="R119" s="9"/>
@@ -8702,7 +8705,7 @@
     </row>
     <row r="120" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A120" s="4" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="B120" s="5">
         <v>46111.53134821759</v>
@@ -8712,16 +8715,16 @@
         <v>46114.628886921295</v>
       </c>
       <c r="E120" s="6" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="F120" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G120" s="6" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="H120" s="6" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="I120" s="6"/>
       <c r="J120" s="5">
@@ -8737,13 +8740,13 @@
         <v>26</v>
       </c>
       <c r="N120" s="6" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="O120" s="6" t="s">
         <v>62</v>
       </c>
       <c r="P120" s="6" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="Q120" s="6"/>
       <c r="R120" s="6"/>
@@ -8753,7 +8756,7 @@
     </row>
     <row r="121" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A121" s="7" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="B121" s="8">
         <v>46111.53139942129</v>
@@ -8769,10 +8772,10 @@
         <v>26</v>
       </c>
       <c r="G121" s="9" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="H121" s="9" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="I121" s="9"/>
       <c r="J121" s="8">
@@ -8788,13 +8791,13 @@
         <v>26</v>
       </c>
       <c r="N121" s="9" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="O121" s="9" t="s">
         <v>65</v>
       </c>
       <c r="P121" s="9" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="Q121" s="9"/>
       <c r="R121" s="9"/>
@@ -8804,7 +8807,7 @@
     </row>
     <row r="122" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A122" s="4" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="B122" s="5">
         <v>46111.53343819444</v>
@@ -8814,16 +8817,16 @@
         <v>46114.628888437495</v>
       </c>
       <c r="E122" s="6" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="F122" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G122" s="6" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="H122" s="6" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="I122" s="6"/>
       <c r="J122" s="5">
@@ -8839,13 +8842,13 @@
         <v>26</v>
       </c>
       <c r="N122" s="6" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="O122" s="6" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="P122" s="6" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="Q122" s="6"/>
       <c r="R122" s="6"/>
@@ -8855,7 +8858,7 @@
     </row>
     <row r="123" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A123" s="7" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="B123" s="8">
         <v>46108.75729289352</v>
@@ -8865,7 +8868,7 @@
         <v>46223.59539700231</v>
       </c>
       <c r="E123" s="9" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="F123" s="9" t="s">
         <v>26</v>
@@ -8892,13 +8895,13 @@
         <v>26</v>
       </c>
       <c r="N123" s="9" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="O123" s="9" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="P123" s="9" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="Q123" s="8">
         <v>46288</v>
@@ -8918,7 +8921,7 @@
     </row>
     <row r="124" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A124" s="4" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="B124" s="5">
         <v>46111.52857409722</v>
@@ -8955,13 +8958,13 @@
         <v>26</v>
       </c>
       <c r="N124" s="6" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="O124" s="6" t="s">
         <v>210</v>
       </c>
       <c r="P124" s="6" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="Q124" s="6"/>
       <c r="R124" s="6"/>
@@ -8971,7 +8974,7 @@
     </row>
     <row r="125" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A125" s="7" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="B125" s="8">
         <v>46111.528674016205</v>
@@ -9008,13 +9011,13 @@
         <v>26</v>
       </c>
       <c r="N125" s="9" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="O125" s="9" t="s">
         <v>215</v>
       </c>
       <c r="P125" s="9" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="Q125" s="9"/>
       <c r="R125" s="9"/>
@@ -9024,7 +9027,7 @@
     </row>
     <row r="126" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A126" s="4" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="B126" s="5">
         <v>46111.531552291664</v>
@@ -9061,13 +9064,13 @@
         <v>26</v>
       </c>
       <c r="N126" s="6" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="O126" s="6" t="s">
         <v>55</v>
       </c>
       <c r="P126" s="6" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="Q126" s="6"/>
       <c r="R126" s="6"/>
@@ -9077,7 +9080,7 @@
     </row>
     <row r="127" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A127" s="7" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="B127" s="8">
         <v>46111.531603344905</v>
@@ -9114,13 +9117,13 @@
         <v>26</v>
       </c>
       <c r="N127" s="9" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="O127" s="9" t="s">
         <v>59</v>
       </c>
       <c r="P127" s="9" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="Q127" s="9"/>
       <c r="R127" s="9"/>
@@ -9130,7 +9133,7 @@
     </row>
     <row r="128" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A128" s="4" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B128" s="5">
         <v>46111.531648379634</v>
@@ -9140,7 +9143,7 @@
         <v>46223.59535668981</v>
       </c>
       <c r="E128" s="6" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="F128" s="6" t="s">
         <v>26</v>
@@ -9167,13 +9170,13 @@
         <v>26</v>
       </c>
       <c r="N128" s="6" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="O128" s="6" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="P128" s="6" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="Q128" s="6"/>
       <c r="R128" s="6"/>
@@ -9183,7 +9186,7 @@
     </row>
     <row r="129" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A129" s="7" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="B129" s="8">
         <v>46111.531705925925</v>
@@ -9220,13 +9223,13 @@
         <v>26</v>
       </c>
       <c r="N129" s="9" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="O129" s="9" t="s">
         <v>65</v>
       </c>
       <c r="P129" s="9" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="Q129" s="9"/>
       <c r="R129" s="9"/>
@@ -9236,7 +9239,7 @@
     </row>
     <row r="130" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A130" s="4" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="B130" s="5">
         <v>46111.533570127314</v>
@@ -9246,7 +9249,7 @@
         <v>46223.59535532407</v>
       </c>
       <c r="E130" s="6" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="F130" s="6" t="s">
         <v>26</v>
@@ -9273,13 +9276,13 @@
         <v>26</v>
       </c>
       <c r="N130" s="6" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="O130" s="6" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="P130" s="6" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="Q130" s="6"/>
       <c r="R130" s="6"/>
@@ -9289,7 +9292,7 @@
     </row>
     <row r="131" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A131" s="7" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="B131" s="8">
         <v>46108.75729930555</v>
@@ -9299,7 +9302,7 @@
         <v>46221.36200443287</v>
       </c>
       <c r="E131" s="9" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="F131" s="9" t="s">
         <v>26</v>
@@ -9326,13 +9329,13 @@
         <v>26</v>
       </c>
       <c r="N131" s="9" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="O131" s="9" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="P131" s="9" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="Q131" s="8">
         <v>46293</v>
@@ -9352,7 +9355,7 @@
     </row>
     <row r="132" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A132" s="4" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="B132" s="5">
         <v>46111.528799872685</v>
@@ -9387,13 +9390,13 @@
         <v>26</v>
       </c>
       <c r="N132" s="6" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="O132" s="6" t="s">
         <v>210</v>
       </c>
       <c r="P132" s="6" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="Q132" s="6"/>
       <c r="R132" s="6"/>
@@ -9403,7 +9406,7 @@
     </row>
     <row r="133" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A133" s="7" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="B133" s="8">
         <v>46111.52885179398</v>
@@ -9438,13 +9441,13 @@
         <v>26</v>
       </c>
       <c r="N133" s="9" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="O133" s="9" t="s">
         <v>215</v>
       </c>
       <c r="P133" s="9" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="Q133" s="9"/>
       <c r="R133" s="9"/>
@@ -9454,7 +9457,7 @@
     </row>
     <row r="134" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A134" s="4" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="B134" s="5">
         <v>46111.53215439815</v>
@@ -9489,13 +9492,13 @@
         <v>26</v>
       </c>
       <c r="N134" s="6" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="O134" s="6" t="s">
         <v>55</v>
       </c>
       <c r="P134" s="6" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="Q134" s="6"/>
       <c r="R134" s="6"/>
@@ -9505,7 +9508,7 @@
     </row>
     <row r="135" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A135" s="7" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="B135" s="8">
         <v>46111.53220642361</v>
@@ -9540,13 +9543,13 @@
         <v>26</v>
       </c>
       <c r="N135" s="9" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="O135" s="9" t="s">
         <v>59</v>
       </c>
       <c r="P135" s="9" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="Q135" s="9"/>
       <c r="R135" s="9"/>
@@ -9556,7 +9559,7 @@
     </row>
     <row r="136" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A136" s="4" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="B136" s="5">
         <v>46111.532258287036</v>
@@ -9566,7 +9569,7 @@
         <v>46114.629316527775</v>
       </c>
       <c r="E136" s="6" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="F136" s="6" t="s">
         <v>26</v>
@@ -9591,13 +9594,13 @@
         <v>26</v>
       </c>
       <c r="N136" s="6" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="O136" s="6" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="P136" s="6" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="Q136" s="6"/>
       <c r="R136" s="6"/>
@@ -9607,7 +9610,7 @@
     </row>
     <row r="137" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A137" s="7" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="B137" s="8">
         <v>46111.53231001158</v>
@@ -9642,13 +9645,13 @@
         <v>26</v>
       </c>
       <c r="N137" s="9" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="O137" s="9" t="s">
         <v>65</v>
       </c>
       <c r="P137" s="9" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="Q137" s="9"/>
       <c r="R137" s="9"/>
@@ -9658,7 +9661,7 @@
     </row>
     <row r="138" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A138" s="4" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="B138" s="5">
         <v>46111.53368237268</v>
@@ -9668,7 +9671,7 @@
         <v>46114.62931805555</v>
       </c>
       <c r="E138" s="6" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="F138" s="6" t="s">
         <v>26</v>
@@ -9693,13 +9696,13 @@
         <v>26</v>
       </c>
       <c r="N138" s="6" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="O138" s="6" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="P138" s="6" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="Q138" s="6"/>
       <c r="R138" s="6"/>
@@ -9709,7 +9712,7 @@
     </row>
     <row r="139" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A139" s="7" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="B139" s="8">
         <v>46108.757304583334</v>
@@ -9719,7 +9722,7 @@
         <v>46240.71896241898</v>
       </c>
       <c r="E139" s="9" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="F139" s="9" t="s">
         <v>26</v>
@@ -9746,13 +9749,13 @@
         <v>26</v>
       </c>
       <c r="N139" s="9" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="O139" s="9" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="P139" s="9" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="Q139" s="8">
         <v>46294</v>
@@ -9772,7 +9775,7 @@
     </row>
     <row r="140" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A140" s="4" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B140" s="5">
         <v>46111.528945011574</v>
@@ -9809,13 +9812,13 @@
         <v>26</v>
       </c>
       <c r="N140" s="6" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="O140" s="6" t="s">
         <v>210</v>
       </c>
       <c r="P140" s="6" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="Q140" s="6"/>
       <c r="R140" s="6"/>
@@ -9825,7 +9828,7 @@
     </row>
     <row r="141" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A141" s="7" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="B141" s="8">
         <v>46111.52901092592</v>
@@ -9862,13 +9865,13 @@
         <v>26</v>
       </c>
       <c r="N141" s="9" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="O141" s="9" t="s">
         <v>215</v>
       </c>
       <c r="P141" s="9" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="Q141" s="9"/>
       <c r="R141" s="9"/>
@@ -9878,7 +9881,7 @@
     </row>
     <row r="142" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A142" s="4" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="B142" s="5">
         <v>46111.53247278935</v>
@@ -9915,13 +9918,13 @@
         <v>26</v>
       </c>
       <c r="N142" s="6" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="O142" s="6" t="s">
         <v>55</v>
       </c>
       <c r="P142" s="6" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="Q142" s="6"/>
       <c r="R142" s="6"/>
@@ -9931,7 +9934,7 @@
     </row>
     <row r="143" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A143" s="7" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="B143" s="8">
         <v>46111.53253350694</v>
@@ -9968,13 +9971,13 @@
         <v>26</v>
       </c>
       <c r="N143" s="9" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="O143" s="9" t="s">
         <v>59</v>
       </c>
       <c r="P143" s="9" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="Q143" s="9"/>
       <c r="R143" s="9"/>
@@ -9984,7 +9987,7 @@
     </row>
     <row r="144" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A144" s="4" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="B144" s="5">
         <v>46111.532638414355</v>
@@ -10021,13 +10024,13 @@
         <v>26</v>
       </c>
       <c r="N144" s="6" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="O144" s="6" t="s">
         <v>65</v>
       </c>
       <c r="P144" s="6" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="Q144" s="6"/>
       <c r="R144" s="6"/>
@@ -10037,7 +10040,7 @@
     </row>
     <row r="145" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A145" s="7" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="B145" s="8">
         <v>46111.53258112269</v>
@@ -10047,7 +10050,7 @@
         <v>46114.83037114583</v>
       </c>
       <c r="E145" s="9" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="F145" s="9" t="s">
         <v>26</v>
@@ -10074,13 +10077,13 @@
         <v>26</v>
       </c>
       <c r="N145" s="9" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="O145" s="9" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="P145" s="9" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="Q145" s="9"/>
       <c r="R145" s="9"/>
@@ -10090,7 +10093,7 @@
     </row>
     <row r="146" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A146" s="4" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="B146" s="5">
         <v>46111.53385627315</v>
@@ -10100,7 +10103,7 @@
         <v>46114.83039427083</v>
       </c>
       <c r="E146" s="6" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="F146" s="6" t="s">
         <v>26</v>
@@ -10127,13 +10130,13 @@
         <v>26</v>
       </c>
       <c r="N146" s="6" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="O146" s="6" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="P146" s="6" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="Q146" s="6"/>
       <c r="R146" s="6"/>
@@ -10143,7 +10146,7 @@
     </row>
     <row r="147" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A147" s="7" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="B147" s="8">
         <v>46108.757310497684</v>
@@ -10153,7 +10156,7 @@
         <v>46114.62962797454</v>
       </c>
       <c r="E147" s="9" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="F147" s="9" t="s">
         <v>25</v>
@@ -10177,7 +10180,7 @@
         <v>26</v>
       </c>
       <c r="O147" s="9" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="P147" s="9" t="s">
         <v>26</v>
@@ -10190,7 +10193,7 @@
     </row>
     <row r="148" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A148" s="4" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="B148" s="5">
         <v>46108.75731366898</v>
@@ -10200,16 +10203,16 @@
         <v>46114.63764361111</v>
       </c>
       <c r="E148" s="6" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="F148" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G148" s="6" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="H148" s="6" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="I148" s="5">
         <v>46295</v>
@@ -10227,13 +10230,13 @@
         <v>26</v>
       </c>
       <c r="N148" s="6" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="O148" s="6" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="P148" s="6" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="Q148" s="5">
         <v>46295</v>
@@ -10253,7 +10256,7 @@
     </row>
     <row r="149" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A149" s="7" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="B149" s="8">
         <v>46108.75732001157</v>
@@ -10263,16 +10266,16 @@
         <v>46119.74841528935</v>
       </c>
       <c r="E149" s="9" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="F149" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G149" s="9" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="H149" s="9" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="I149" s="8">
         <v>46295</v>
@@ -10290,13 +10293,13 @@
         <v>26</v>
       </c>
       <c r="N149" s="9" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="O149" s="9" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="P149" s="9" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="Q149" s="8">
         <v>46295</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-08-28 13:46 UTC
</commit_message>
<xml_diff>
--- a/data/50001525 - ZITRON PERU METRO LIMA E07.xlsx
+++ b/data/50001525 - ZITRON PERU METRO LIMA E07.xlsx
@@ -7429,7 +7429,7 @@
       </c>
       <c r="C96" s="6"/>
       <c r="D96" s="5">
-        <v>46223.595235995366</v>
+        <v>46262.17811915509</v>
       </c>
       <c r="E96" s="6" t="s">
         <v>319</v>
@@ -7476,8 +7476,8 @@
       <c r="S96" s="6">
         <v>0</v>
       </c>
-      <c r="T96" s="11" t="s">
-        <v>127</v>
+      <c r="T96" s="12" t="s">
+        <v>311</v>
       </c>
       <c r="U96" s="10" t="s">
         <v>53</v>

</xml_diff>

<commit_message>
Actualizacion automatica 2026-09-02 17:10 UTC
</commit_message>
<xml_diff>
--- a/data/50001525 - ZITRON PERU METRO LIMA E07.xlsx
+++ b/data/50001525 - ZITRON PERU METRO LIMA E07.xlsx
@@ -6963,7 +6963,7 @@
       </c>
       <c r="C88" s="6"/>
       <c r="D88" s="5">
-        <v>46111.59782981481</v>
+        <v>46267.17843465278</v>
       </c>
       <c r="E88" s="6" t="s">
         <v>298</v>
@@ -7010,8 +7010,8 @@
       <c r="S88" s="6">
         <v>0</v>
       </c>
-      <c r="T88" s="11" t="s">
-        <v>127</v>
+      <c r="T88" s="12" t="s">
+        <v>152</v>
       </c>
       <c r="U88" s="10" t="s">
         <v>53</v>
@@ -7260,7 +7260,7 @@
       </c>
       <c r="C93" s="9"/>
       <c r="D93" s="8">
-        <v>46260.19028297454</v>
+        <v>46267.16748222223</v>
       </c>
       <c r="E93" s="9" t="s">
         <v>311</v>
@@ -7323,7 +7323,7 @@
       </c>
       <c r="C94" s="6"/>
       <c r="D94" s="5">
-        <v>46260.577836412034</v>
+        <v>46267.167487708335</v>
       </c>
       <c r="E94" s="6" t="s">
         <v>211</v>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="C95" s="9"/>
       <c r="D95" s="8">
-        <v>46260.57785292824</v>
+        <v>46267.167488796294</v>
       </c>
       <c r="E95" s="9" t="s">
         <v>216</v>

</xml_diff>

<commit_message>
Actualizacion automatica 2026-09-04 16:56 UTC
</commit_message>
<xml_diff>
--- a/data/50001525 - ZITRON PERU METRO LIMA E07.xlsx
+++ b/data/50001525 - ZITRON PERU METRO LIMA E07.xlsx
@@ -7429,7 +7429,7 @@
       </c>
       <c r="C96" s="6"/>
       <c r="D96" s="5">
-        <v>46262.17811915509</v>
+        <v>46269.16768288195</v>
       </c>
       <c r="E96" s="6" t="s">
         <v>319</v>
@@ -7492,7 +7492,7 @@
       </c>
       <c r="C97" s="9"/>
       <c r="D97" s="8">
-        <v>46227.72251041667</v>
+        <v>46269.167690648144</v>
       </c>
       <c r="E97" s="9" t="s">
         <v>211</v>
@@ -7545,7 +7545,7 @@
       </c>
       <c r="C98" s="6"/>
       <c r="D98" s="5">
-        <v>46227.72251091435</v>
+        <v>46269.16769188657</v>
       </c>
       <c r="E98" s="6" t="s">
         <v>216</v>

</xml_diff>

<commit_message>
Curva S actualizada 2026-09-05 12:03 Chile
</commit_message>
<xml_diff>
--- a/data/50001525 - ZITRON PERU METRO LIMA E07.xlsx
+++ b/data/50001525 - ZITRON PERU METRO LIMA E07.xlsx
@@ -7429,7 +7429,7 @@
       </c>
       <c r="C96" s="6"/>
       <c r="D96" s="5">
-        <v>46269.16768288195</v>
+        <v>46270.18529125</v>
       </c>
       <c r="E96" s="6" t="s">
         <v>319</v>
@@ -7476,8 +7476,8 @@
       <c r="S96" s="6">
         <v>0</v>
       </c>
-      <c r="T96" s="12" t="s">
-        <v>152</v>
+      <c r="T96" s="10" t="s">
+        <v>31</v>
       </c>
       <c r="U96" s="10" t="s">
         <v>53</v>

</xml_diff>

<commit_message>
Actualizacion automatica 2026-09-08 17:12 UTC
</commit_message>
<xml_diff>
--- a/data/50001525 - ZITRON PERU METRO LIMA E07.xlsx
+++ b/data/50001525 - ZITRON PERU METRO LIMA E07.xlsx
@@ -469,445 +469,445 @@
     <t>Generación OC motor ot 4287 - 4288,Fabricación motor ot 4287 - 4288,Planos motor proveedor ot 4287 - 4288</t>
   </si>
   <si>
+    <t>1213833564682558</t>
+  </si>
+  <si>
+    <t>Generación OC motor ot 4287 - 4288</t>
+  </si>
+  <si>
+    <t>Generación OC motor,Motor ot 4287 - 4288,Fabricación motor ot 4287 - 4288,Planos motor proveedor ot 4287 - 4288</t>
+  </si>
+  <si>
+    <t>1213833564685848</t>
+  </si>
+  <si>
+    <t>Fabricación motor ot 4287 - 4288</t>
+  </si>
+  <si>
+    <t>Motor ot 4287 - 4288,Recepcion motor</t>
+  </si>
+  <si>
+    <t>1213833564685869</t>
+  </si>
+  <si>
+    <t>Planos motor proveedor ot 4287 - 4288</t>
+  </si>
+  <si>
+    <t>Motor ot 4287 - 4288,OT 4287 ZVR 1-14-42/4,OT 4288 ZVR1-14-30/4</t>
+  </si>
+  <si>
+    <t>1213833777483152</t>
+  </si>
+  <si>
+    <t>Materiales a codigo // compras locales aprovisionamientomiento: ot 4287 - 4288</t>
+  </si>
+  <si>
+    <t>Yerlia Ayleen Castillo Diaz</t>
+  </si>
+  <si>
+    <t>yerlia.castillo@zitron.com</t>
+  </si>
+  <si>
+    <t>Generación OC materiales ot 4287 - 4288,Fabricacion a codigo y compras locales ot 4287 - 4288</t>
+  </si>
+  <si>
+    <t>1213833777483168</t>
+  </si>
+  <si>
+    <t>Materiales a codigo // compras locales aprovisionamientomiento: ot 4287 - 4288,Fabricacion a codigo y compras locales ot 4287 - 4288</t>
+  </si>
+  <si>
+    <t>1213833564688412</t>
+  </si>
+  <si>
+    <t>Fabricacion a codigo y compras locales ot 4287 - 4288</t>
+  </si>
+  <si>
+    <t>Materiales a codigo // compras locales aprovisionamientomiento: ot 4287 - 4288,Recepcion materiales a codigos // compras locales aprovisionamiento,Fabricacion estructura proveedor externo ot 4287 - 4288</t>
+  </si>
+  <si>
+    <t>1213833763284961</t>
+  </si>
+  <si>
+    <t>Sensores</t>
+  </si>
+  <si>
+    <t>Generacion OC Sensor,Fabricacion Sensores</t>
+  </si>
+  <si>
+    <t>1213833763284977</t>
+  </si>
+  <si>
+    <t>Generacion OC Sensor</t>
+  </si>
+  <si>
+    <t>Sensores,Fabricacion Sensores</t>
+  </si>
+  <si>
+    <t>1213833777489751</t>
+  </si>
+  <si>
+    <t>Fabricacion Sensores</t>
+  </si>
+  <si>
+    <t>Recepción Sensores,Sensores</t>
+  </si>
+  <si>
+    <t>1213833777489767</t>
+  </si>
+  <si>
+    <t>Fabricacion Externa ot 4287 - 4288</t>
+  </si>
+  <si>
+    <t>Rosemary Singh</t>
+  </si>
+  <si>
+    <t>rosemary.singh@zitron.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Generacion OC Fabricacion Externa ot 4287 - 4288,Fabricacion estructura proveedor externo ot 4287 - 4288</t>
+  </si>
+  <si>
+    <t>1213833564667630</t>
+  </si>
+  <si>
+    <t>Fabricacion Externa ot 4287 - 4288,Fabricacion estructura proveedor externo ot 4287 - 4288</t>
+  </si>
+  <si>
+    <t>1213833763295351</t>
+  </si>
+  <si>
+    <t>Fabricacion estructura proveedor externo ot 4287 - 4288</t>
+  </si>
+  <si>
+    <t>Check Planos,Fabricacion a codigo y compras locales ot 4287 - 4288, Generacion OC Fabricacion Externa ot 4287 - 4288</t>
+  </si>
+  <si>
+    <t>Control de calidad Fabricación externa,Fabricacion Externa ot 4287 - 4288</t>
+  </si>
+  <si>
+    <t>1213869987281796</t>
+  </si>
+  <si>
+    <t>Atenuador ot 4289</t>
+  </si>
+  <si>
+    <t>Propuesta Atenuadores ,Generacion oc Atenuador  ot 4289,Fabricacion atenuador ot 4289</t>
+  </si>
+  <si>
+    <t>1213869987281797</t>
+  </si>
+  <si>
+    <t>Generacion oc Atenuador  ot 4289</t>
+  </si>
+  <si>
+    <t>Fabricacion atenuador ot 4289,Atenuador ot 4289</t>
+  </si>
+  <si>
+    <t>1213869987281798</t>
+  </si>
+  <si>
+    <t>Fabricacion atenuador ot 4289</t>
+  </si>
+  <si>
+    <t>Atenuadores,Atenuador ot 4289</t>
+  </si>
+  <si>
+    <t>1213833564706217</t>
+  </si>
+  <si>
+    <t>Ingenieria y diseño:</t>
+  </si>
+  <si>
+    <t>Planos preliminar,Planos definitivos</t>
+  </si>
+  <si>
+    <t>1213833564706230</t>
+  </si>
+  <si>
+    <t>Planos preliminar</t>
+  </si>
+  <si>
+    <t>Gonzalo Javier Dávila Bade</t>
+  </si>
+  <si>
+    <t>gonzalo.davila@zitron.com</t>
+  </si>
+  <si>
+    <t>Ingenieria Detalle,OT 4287 ZVR 1-14-42/4,OT 4288 ZVR1-14-30/4</t>
+  </si>
+  <si>
+    <t>Ingenieria y diseño:,Check Planos</t>
+  </si>
+  <si>
+    <t>1213899500210867</t>
+  </si>
+  <si>
+    <t>OT 4287 ZVR 1-14-42/4</t>
+  </si>
+  <si>
+    <t>Hernan Roberto Gutierrez Barrientos</t>
+  </si>
+  <si>
+    <t>hgutierrez@zitron.com</t>
+  </si>
+  <si>
+    <t>Planos preliminar,OT 4287 ZVR 1-14-42/4</t>
+  </si>
+  <si>
+    <t>1213899500210869</t>
+  </si>
+  <si>
+    <t>OT 4288 ZVR1-14-30/4</t>
+  </si>
+  <si>
+    <t>Planos preliminar,OT 4288 ZVR1-14-30/4</t>
+  </si>
+  <si>
+    <t>1213833763300853</t>
+  </si>
+  <si>
+    <t>Planos definitivos</t>
+  </si>
+  <si>
+    <t>OT 4287 ZVR 1-14-42/4,OT 4288 ZVR1-14-30/4</t>
+  </si>
+  <si>
+    <t>Check Planos,Ingenieria y diseño:</t>
+  </si>
+  <si>
+    <t>1213899500210870</t>
+  </si>
+  <si>
+    <t>OT 4287 ZVR 1-14-42/4,Planos motor proveedor ot 4287 - 4288</t>
+  </si>
+  <si>
+    <t>Planos definitivos,OT 4287 ZVR 1-14-42/4</t>
+  </si>
+  <si>
+    <t>1213899500210871</t>
+  </si>
+  <si>
+    <t>OT 4288 ZVR1-14-30/4,Planos motor proveedor ot 4287 - 4288</t>
+  </si>
+  <si>
+    <t>Planos definitivos,OT4288 ZVR1-14-30/4</t>
+  </si>
+  <si>
+    <t>1213833763300879</t>
+  </si>
+  <si>
+    <t>Planos definitivos,Planos preliminar</t>
+  </si>
+  <si>
+    <t>OT 4287 ZVR 1-14-42/4,OT 4288 ZVR1-14-30/4,OT 4287 ZVR 1-14-42/4,OT 4288 ZVR1-14-30/4,OT 4287 ZVR 1-14-42/4,OT 4288 ZVR1-14-30/4,OT 4288 ZVR1-14-30/4,OT 4287 ZVR 1-14-42/4,OT 4288 ZVR1-14-30/4,OT 4287 ZVR 1-14-42/4,OT 4288 ZVR1-14-30/4,OT 4287 ZVR 1-14-42/4,propuesta compras a codigo // aprovisionamiento ot 4287 - 4288,Propuesta Fabricacion Externa ot 4287 - 4288,Fabricacion estructura proveedor externo ot 4287 - 4288</t>
+  </si>
+  <si>
+    <t>1213899500210872</t>
+  </si>
+  <si>
+    <t>1213899500210873</t>
+  </si>
+  <si>
+    <t>OT4288 ZVR1-14-30/4</t>
+  </si>
+  <si>
+    <t>1213833622855505</t>
+  </si>
+  <si>
+    <t>Check pruebas FAT</t>
+  </si>
+  <si>
+    <t>Francisca González Cornejo</t>
+  </si>
+  <si>
+    <t>francisca.gonzalez@zitron.com</t>
+  </si>
+  <si>
+    <t>OT 4287 ZVR 1-14-42/4,OT  4288 ZVR1-14-30/4</t>
+  </si>
+  <si>
+    <t>1213869987281952</t>
+  </si>
+  <si>
+    <t>Check pruebas FAT,OT 4287 ZVR 1-14-42/4</t>
+  </si>
+  <si>
+    <t>1213869987281953</t>
+  </si>
+  <si>
+    <t>OT  4288 ZVR1-14-30/4</t>
+  </si>
+  <si>
+    <t>Check pruebas FAT,OT 4288 ZVR1-14-30/4</t>
+  </si>
+  <si>
+    <t>1213833622855516</t>
+  </si>
+  <si>
+    <t>Control de calidad</t>
+  </si>
+  <si>
+    <t>Control de calidad Fabricación externa</t>
+  </si>
+  <si>
+    <t>1213833622855625</t>
+  </si>
+  <si>
+    <t>Nicolás López</t>
+  </si>
+  <si>
+    <t>nicolas.lopez@zitron.com</t>
+  </si>
+  <si>
+    <t>Control de calidad,Recepcion Fabricacion externa</t>
+  </si>
+  <si>
+    <t>1213840446207872</t>
+  </si>
+  <si>
+    <t>Bodega</t>
+  </si>
+  <si>
+    <t>Recepcion materiales a codigos // compras locales aprovisionamiento,Control de calidad compras materiales a codigo // compras locale aprovisionamient</t>
+  </si>
+  <si>
+    <t>1213840446207876</t>
+  </si>
+  <si>
+    <t>Recepcion materiales a codigos // compras locales aprovisionamiento</t>
+  </si>
+  <si>
+    <t>Victor Muñoz</t>
+  </si>
+  <si>
+    <t>victor.munoz@zitron.com</t>
+  </si>
+  <si>
+    <t>Control de calidad compras materiales a codigo // compras locale aprovisionamient,Bodega</t>
+  </si>
+  <si>
+    <t>1213840446207878</t>
+  </si>
+  <si>
+    <t>Control de calidad compras materiales a codigo // compras locale aprovisionamient</t>
+  </si>
+  <si>
+    <t>Bodega,Preparacion materiales</t>
+  </si>
+  <si>
+    <t>1213869987281780</t>
+  </si>
+  <si>
+    <t>Caldereria</t>
+  </si>
+  <si>
+    <t>Preparacion materiales,Armado,Control de calidad Armado</t>
+  </si>
+  <si>
+    <t>1213869987281782</t>
+  </si>
+  <si>
+    <t>Preparacion materiales</t>
+  </si>
+  <si>
+    <t>Nicolás Mol</t>
+  </si>
+  <si>
+    <t>nicolas.mol@zitron.com</t>
+  </si>
+  <si>
+    <t>Caldereria,OT 4287 ZVR 1-14-42/4,OT 4288 ZVR1-14-30/4</t>
+  </si>
+  <si>
+    <t>1213869987281784</t>
+  </si>
+  <si>
+    <t>Armado</t>
+  </si>
+  <si>
+    <t>Caldereria,Control de calidad Armado  4388</t>
+  </si>
+  <si>
+    <t>1213869987281817</t>
+  </si>
+  <si>
+    <t>Preparacion materiales,Check Planos</t>
+  </si>
+  <si>
+    <t>Armado,OT 4287 ZVR 1-14-42/4</t>
+  </si>
+  <si>
+    <t>1213869987281819</t>
+  </si>
+  <si>
+    <t>Armado,OT 4288 ZVR1-14-30/4</t>
+  </si>
+  <si>
+    <t>1213869987281786</t>
+  </si>
+  <si>
+    <t>Control de calidad Armado</t>
+  </si>
+  <si>
+    <t>1213869987281820</t>
+  </si>
+  <si>
+    <t>OT 4287 ZVR 1-14-42/4,Check Planos</t>
+  </si>
+  <si>
+    <t>Control de calidad Armado,OT 4287 ZVR 1-14-42/4</t>
+  </si>
+  <si>
+    <t>1213869987281821</t>
+  </si>
+  <si>
+    <t>OT 4288 ZVR1-14-30/4,Check Planos</t>
+  </si>
+  <si>
+    <t>Control de calidad Armado,OT 4288 ZVR1-14-30/4</t>
+  </si>
+  <si>
+    <t>1213833622855646</t>
+  </si>
+  <si>
+    <t>Bodega:</t>
+  </si>
+  <si>
+    <t>Recepcion Alabe,Recepcion motor,Recepcion Fabricacion externa,Recepcion Rodete,Recepcion Tableros y componentes electricos</t>
+  </si>
+  <si>
+    <t>1213833763304341</t>
+  </si>
+  <si>
+    <t>Recepcion Rodete</t>
+  </si>
+  <si>
+    <t>Bodega:,OT 4287 ZVR 1-14-42/4,OT 4288 ZVR1-14-30/4</t>
+  </si>
+  <si>
+    <t>1213833763304362</t>
+  </si>
+  <si>
+    <t>Bodega:,OT 4290 - TABLERO VDF ABB ACS880-17,OT 4291- TABLERO PLC,OT 4292- TABLERO BOTONERA ,OT 4293-COMPONENTES TABLERO COMPUERTAS</t>
+  </si>
+  <si>
+    <t>1213833806791953</t>
+  </si>
+  <si>
+    <t>Recepcion Alabe</t>
+  </si>
+  <si>
+    <t>Bodega:,OT 4288 ZVR1-14-30/4,OT 4287 ZVR 1-14-42/4</t>
+  </si>
+  <si>
+    <t>1213833564712053</t>
+  </si>
+  <si>
+    <t>Recepcion motor</t>
+  </si>
+  <si>
     <t>Media</t>
-  </si>
-  <si>
-    <t>1213833564682558</t>
-  </si>
-  <si>
-    <t>Generación OC motor ot 4287 - 4288</t>
-  </si>
-  <si>
-    <t>Generación OC motor,Motor ot 4287 - 4288,Fabricación motor ot 4287 - 4288,Planos motor proveedor ot 4287 - 4288</t>
-  </si>
-  <si>
-    <t>1213833564685848</t>
-  </si>
-  <si>
-    <t>Fabricación motor ot 4287 - 4288</t>
-  </si>
-  <si>
-    <t>Motor ot 4287 - 4288,Recepcion motor</t>
-  </si>
-  <si>
-    <t>1213833564685869</t>
-  </si>
-  <si>
-    <t>Planos motor proveedor ot 4287 - 4288</t>
-  </si>
-  <si>
-    <t>Motor ot 4287 - 4288,OT 4287 ZVR 1-14-42/4,OT 4288 ZVR1-14-30/4</t>
-  </si>
-  <si>
-    <t>1213833777483152</t>
-  </si>
-  <si>
-    <t>Materiales a codigo // compras locales aprovisionamientomiento: ot 4287 - 4288</t>
-  </si>
-  <si>
-    <t>Yerlia Ayleen Castillo Diaz</t>
-  </si>
-  <si>
-    <t>yerlia.castillo@zitron.com</t>
-  </si>
-  <si>
-    <t>Generación OC materiales ot 4287 - 4288,Fabricacion a codigo y compras locales ot 4287 - 4288</t>
-  </si>
-  <si>
-    <t>1213833777483168</t>
-  </si>
-  <si>
-    <t>Materiales a codigo // compras locales aprovisionamientomiento: ot 4287 - 4288,Fabricacion a codigo y compras locales ot 4287 - 4288</t>
-  </si>
-  <si>
-    <t>1213833564688412</t>
-  </si>
-  <si>
-    <t>Fabricacion a codigo y compras locales ot 4287 - 4288</t>
-  </si>
-  <si>
-    <t>Materiales a codigo // compras locales aprovisionamientomiento: ot 4287 - 4288,Recepcion materiales a codigos // compras locales aprovisionamiento,Fabricacion estructura proveedor externo ot 4287 - 4288</t>
-  </si>
-  <si>
-    <t>1213833763284961</t>
-  </si>
-  <si>
-    <t>Sensores</t>
-  </si>
-  <si>
-    <t>Generacion OC Sensor,Fabricacion Sensores</t>
-  </si>
-  <si>
-    <t>1213833763284977</t>
-  </si>
-  <si>
-    <t>Generacion OC Sensor</t>
-  </si>
-  <si>
-    <t>Sensores,Fabricacion Sensores</t>
-  </si>
-  <si>
-    <t>1213833777489751</t>
-  </si>
-  <si>
-    <t>Fabricacion Sensores</t>
-  </si>
-  <si>
-    <t>Recepción Sensores,Sensores</t>
-  </si>
-  <si>
-    <t>1213833777489767</t>
-  </si>
-  <si>
-    <t>Fabricacion Externa ot 4287 - 4288</t>
-  </si>
-  <si>
-    <t>Rosemary Singh</t>
-  </si>
-  <si>
-    <t>rosemary.singh@zitron.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Generacion OC Fabricacion Externa ot 4287 - 4288,Fabricacion estructura proveedor externo ot 4287 - 4288</t>
-  </si>
-  <si>
-    <t>1213833564667630</t>
-  </si>
-  <si>
-    <t>Fabricacion Externa ot 4287 - 4288,Fabricacion estructura proveedor externo ot 4287 - 4288</t>
-  </si>
-  <si>
-    <t>1213833763295351</t>
-  </si>
-  <si>
-    <t>Fabricacion estructura proveedor externo ot 4287 - 4288</t>
-  </si>
-  <si>
-    <t>Check Planos,Fabricacion a codigo y compras locales ot 4287 - 4288, Generacion OC Fabricacion Externa ot 4287 - 4288</t>
-  </si>
-  <si>
-    <t>Control de calidad Fabricación externa,Fabricacion Externa ot 4287 - 4288</t>
-  </si>
-  <si>
-    <t>1213869987281796</t>
-  </si>
-  <si>
-    <t>Atenuador ot 4289</t>
-  </si>
-  <si>
-    <t>Propuesta Atenuadores ,Generacion oc Atenuador  ot 4289,Fabricacion atenuador ot 4289</t>
-  </si>
-  <si>
-    <t>1213869987281797</t>
-  </si>
-  <si>
-    <t>Generacion oc Atenuador  ot 4289</t>
-  </si>
-  <si>
-    <t>Fabricacion atenuador ot 4289,Atenuador ot 4289</t>
-  </si>
-  <si>
-    <t>1213869987281798</t>
-  </si>
-  <si>
-    <t>Fabricacion atenuador ot 4289</t>
-  </si>
-  <si>
-    <t>Atenuadores,Atenuador ot 4289</t>
-  </si>
-  <si>
-    <t>1213833564706217</t>
-  </si>
-  <si>
-    <t>Ingenieria y diseño:</t>
-  </si>
-  <si>
-    <t>Planos preliminar,Planos definitivos</t>
-  </si>
-  <si>
-    <t>1213833564706230</t>
-  </si>
-  <si>
-    <t>Planos preliminar</t>
-  </si>
-  <si>
-    <t>Gonzalo Javier Dávila Bade</t>
-  </si>
-  <si>
-    <t>gonzalo.davila@zitron.com</t>
-  </si>
-  <si>
-    <t>Ingenieria Detalle,OT 4287 ZVR 1-14-42/4,OT 4288 ZVR1-14-30/4</t>
-  </si>
-  <si>
-    <t>Ingenieria y diseño:,Check Planos</t>
-  </si>
-  <si>
-    <t>1213899500210867</t>
-  </si>
-  <si>
-    <t>OT 4287 ZVR 1-14-42/4</t>
-  </si>
-  <si>
-    <t>Hernan Roberto Gutierrez Barrientos</t>
-  </si>
-  <si>
-    <t>hgutierrez@zitron.com</t>
-  </si>
-  <si>
-    <t>Planos preliminar,OT 4287 ZVR 1-14-42/4</t>
-  </si>
-  <si>
-    <t>1213899500210869</t>
-  </si>
-  <si>
-    <t>OT 4288 ZVR1-14-30/4</t>
-  </si>
-  <si>
-    <t>Planos preliminar,OT 4288 ZVR1-14-30/4</t>
-  </si>
-  <si>
-    <t>1213833763300853</t>
-  </si>
-  <si>
-    <t>Planos definitivos</t>
-  </si>
-  <si>
-    <t>OT 4287 ZVR 1-14-42/4,OT 4288 ZVR1-14-30/4</t>
-  </si>
-  <si>
-    <t>Check Planos,Ingenieria y diseño:</t>
-  </si>
-  <si>
-    <t>1213899500210870</t>
-  </si>
-  <si>
-    <t>OT 4287 ZVR 1-14-42/4,Planos motor proveedor ot 4287 - 4288</t>
-  </si>
-  <si>
-    <t>Planos definitivos,OT 4287 ZVR 1-14-42/4</t>
-  </si>
-  <si>
-    <t>1213899500210871</t>
-  </si>
-  <si>
-    <t>OT 4288 ZVR1-14-30/4,Planos motor proveedor ot 4287 - 4288</t>
-  </si>
-  <si>
-    <t>Planos definitivos,OT4288 ZVR1-14-30/4</t>
-  </si>
-  <si>
-    <t>1213833763300879</t>
-  </si>
-  <si>
-    <t>Planos definitivos,Planos preliminar</t>
-  </si>
-  <si>
-    <t>OT 4287 ZVR 1-14-42/4,OT 4288 ZVR1-14-30/4,OT 4287 ZVR 1-14-42/4,OT 4288 ZVR1-14-30/4,OT 4287 ZVR 1-14-42/4,OT 4288 ZVR1-14-30/4,OT 4288 ZVR1-14-30/4,OT 4287 ZVR 1-14-42/4,OT 4288 ZVR1-14-30/4,OT 4287 ZVR 1-14-42/4,OT 4288 ZVR1-14-30/4,OT 4287 ZVR 1-14-42/4,propuesta compras a codigo // aprovisionamiento ot 4287 - 4288,Propuesta Fabricacion Externa ot 4287 - 4288,Fabricacion estructura proveedor externo ot 4287 - 4288</t>
-  </si>
-  <si>
-    <t>1213899500210872</t>
-  </si>
-  <si>
-    <t>1213899500210873</t>
-  </si>
-  <si>
-    <t>OT4288 ZVR1-14-30/4</t>
-  </si>
-  <si>
-    <t>1213833622855505</t>
-  </si>
-  <si>
-    <t>Check pruebas FAT</t>
-  </si>
-  <si>
-    <t>Francisca González Cornejo</t>
-  </si>
-  <si>
-    <t>francisca.gonzalez@zitron.com</t>
-  </si>
-  <si>
-    <t>OT 4287 ZVR 1-14-42/4,OT  4288 ZVR1-14-30/4</t>
-  </si>
-  <si>
-    <t>1213869987281952</t>
-  </si>
-  <si>
-    <t>Check pruebas FAT,OT 4287 ZVR 1-14-42/4</t>
-  </si>
-  <si>
-    <t>1213869987281953</t>
-  </si>
-  <si>
-    <t>OT  4288 ZVR1-14-30/4</t>
-  </si>
-  <si>
-    <t>Check pruebas FAT,OT 4288 ZVR1-14-30/4</t>
-  </si>
-  <si>
-    <t>1213833622855516</t>
-  </si>
-  <si>
-    <t>Control de calidad</t>
-  </si>
-  <si>
-    <t>Control de calidad Fabricación externa</t>
-  </si>
-  <si>
-    <t>1213833622855625</t>
-  </si>
-  <si>
-    <t>Nicolás López</t>
-  </si>
-  <si>
-    <t>nicolas.lopez@zitron.com</t>
-  </si>
-  <si>
-    <t>Control de calidad,Recepcion Fabricacion externa</t>
-  </si>
-  <si>
-    <t>1213840446207872</t>
-  </si>
-  <si>
-    <t>Bodega</t>
-  </si>
-  <si>
-    <t>Recepcion materiales a codigos // compras locales aprovisionamiento,Control de calidad compras materiales a codigo // compras locale aprovisionamient</t>
-  </si>
-  <si>
-    <t>1213840446207876</t>
-  </si>
-  <si>
-    <t>Recepcion materiales a codigos // compras locales aprovisionamiento</t>
-  </si>
-  <si>
-    <t>Victor Muñoz</t>
-  </si>
-  <si>
-    <t>victor.munoz@zitron.com</t>
-  </si>
-  <si>
-    <t>Control de calidad compras materiales a codigo // compras locale aprovisionamient,Bodega</t>
-  </si>
-  <si>
-    <t>1213840446207878</t>
-  </si>
-  <si>
-    <t>Control de calidad compras materiales a codigo // compras locale aprovisionamient</t>
-  </si>
-  <si>
-    <t>Bodega,Preparacion materiales</t>
-  </si>
-  <si>
-    <t>1213869987281780</t>
-  </si>
-  <si>
-    <t>Caldereria</t>
-  </si>
-  <si>
-    <t>Preparacion materiales,Armado,Control de calidad Armado</t>
-  </si>
-  <si>
-    <t>1213869987281782</t>
-  </si>
-  <si>
-    <t>Preparacion materiales</t>
-  </si>
-  <si>
-    <t>Nicolás Mol</t>
-  </si>
-  <si>
-    <t>nicolas.mol@zitron.com</t>
-  </si>
-  <si>
-    <t>Caldereria,OT 4287 ZVR 1-14-42/4,OT 4288 ZVR1-14-30/4</t>
-  </si>
-  <si>
-    <t>1213869987281784</t>
-  </si>
-  <si>
-    <t>Armado</t>
-  </si>
-  <si>
-    <t>Caldereria,Control de calidad Armado  4388</t>
-  </si>
-  <si>
-    <t>1213869987281817</t>
-  </si>
-  <si>
-    <t>Preparacion materiales,Check Planos</t>
-  </si>
-  <si>
-    <t>Armado,OT 4287 ZVR 1-14-42/4</t>
-  </si>
-  <si>
-    <t>1213869987281819</t>
-  </si>
-  <si>
-    <t>Armado,OT 4288 ZVR1-14-30/4</t>
-  </si>
-  <si>
-    <t>1213869987281786</t>
-  </si>
-  <si>
-    <t>Control de calidad Armado</t>
-  </si>
-  <si>
-    <t>1213869987281820</t>
-  </si>
-  <si>
-    <t>OT 4287 ZVR 1-14-42/4,Check Planos</t>
-  </si>
-  <si>
-    <t>Control de calidad Armado,OT 4287 ZVR 1-14-42/4</t>
-  </si>
-  <si>
-    <t>1213869987281821</t>
-  </si>
-  <si>
-    <t>OT 4288 ZVR1-14-30/4,Check Planos</t>
-  </si>
-  <si>
-    <t>Control de calidad Armado,OT 4288 ZVR1-14-30/4</t>
-  </si>
-  <si>
-    <t>1213833622855646</t>
-  </si>
-  <si>
-    <t>Bodega:</t>
-  </si>
-  <si>
-    <t>Recepcion Alabe,Recepcion motor,Recepcion Fabricacion externa,Recepcion Rodete,Recepcion Tableros y componentes electricos</t>
-  </si>
-  <si>
-    <t>1213833763304341</t>
-  </si>
-  <si>
-    <t>Recepcion Rodete</t>
-  </si>
-  <si>
-    <t>Bodega:,OT 4287 ZVR 1-14-42/4,OT 4288 ZVR1-14-30/4</t>
-  </si>
-  <si>
-    <t>1213833763304362</t>
-  </si>
-  <si>
-    <t>Bodega:,OT 4290 - TABLERO VDF ABB ACS880-17,OT 4291- TABLERO PLC,OT 4292- TABLERO BOTONERA ,OT 4293-COMPONENTES TABLERO COMPUERTAS</t>
-  </si>
-  <si>
-    <t>1213833806791953</t>
-  </si>
-  <si>
-    <t>Recepcion Alabe</t>
-  </si>
-  <si>
-    <t>Bodega:,OT 4288 ZVR1-14-30/4,OT 4287 ZVR 1-14-42/4</t>
-  </si>
-  <si>
-    <t>1213833564712053</t>
-  </si>
-  <si>
-    <t>Recepcion motor</t>
   </si>
   <si>
     <t>1213833564713244</t>
@@ -4267,7 +4267,7 @@
       </c>
       <c r="C42" s="6"/>
       <c r="D42" s="5">
-        <v>46272.16711635416</v>
+        <v>46273.135429918984</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>150</v>
@@ -4314,8 +4314,8 @@
       <c r="S42" s="6">
         <v>0</v>
       </c>
-      <c r="T42" s="12" t="s">
-        <v>152</v>
+      <c r="T42" s="10" t="s">
+        <v>31</v>
       </c>
       <c r="U42" s="10" t="s">
         <v>53</v>
@@ -4323,7 +4323,7 @@
     </row>
     <row r="43" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A43" s="7" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B43" s="8">
         <v>46108.75700856482</v>
@@ -4335,7 +4335,7 @@
         <v>46182.69343975694</v>
       </c>
       <c r="E43" s="9" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F43" s="9" t="s">
         <v>26</v>
@@ -4368,7 +4368,7 @@
         <v>91</v>
       </c>
       <c r="P43" s="9" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="Q43" s="8">
         <v>45978</v>
@@ -4388,7 +4388,7 @@
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B44" s="5">
         <v>46108.757016435186</v>
@@ -4398,7 +4398,7 @@
         <v>46272.16711458333</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="F44" s="6" t="s">
         <v>26</v>
@@ -4428,10 +4428,10 @@
         <v>150</v>
       </c>
       <c r="O44" s="6" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="P44" s="6" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="Q44" s="5">
         <v>45999</v>
@@ -4451,7 +4451,7 @@
     </row>
     <row r="45" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A45" s="7" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B45" s="8">
         <v>46108.7570218287</v>
@@ -4463,7 +4463,7 @@
         <v>46211.84652803241</v>
       </c>
       <c r="E45" s="9" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F45" s="9" t="s">
         <v>26</v>
@@ -4493,10 +4493,10 @@
         <v>150</v>
       </c>
       <c r="O45" s="9" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="P45" s="9" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="Q45" s="8">
         <v>45999</v>
@@ -4516,7 +4516,7 @@
     </row>
     <row r="46" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B46" s="5">
         <v>46108.75702719907</v>
@@ -4528,16 +4528,16 @@
         <v>46260.58088763889</v>
       </c>
       <c r="E46" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="F46" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G46" s="6" t="s">
         <v>163</v>
       </c>
-      <c r="F46" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G46" s="6" t="s">
+      <c r="H46" s="6" t="s">
         <v>164</v>
-      </c>
-      <c r="H46" s="6" t="s">
-        <v>165</v>
       </c>
       <c r="I46" s="5">
         <v>46195</v>
@@ -4558,7 +4558,7 @@
         <v>117</v>
       </c>
       <c r="O46" s="6" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="P46" s="6" t="s">
         <v>117</v>
@@ -4581,7 +4581,7 @@
     </row>
     <row r="47" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A47" s="7" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B47" s="8">
         <v>46108.75703201389</v>
@@ -4599,10 +4599,10 @@
         <v>26</v>
       </c>
       <c r="G47" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="H47" s="9" t="s">
         <v>164</v>
-      </c>
-      <c r="H47" s="9" t="s">
-        <v>165</v>
       </c>
       <c r="I47" s="8">
         <v>46195</v>
@@ -4620,13 +4620,13 @@
         <v>26</v>
       </c>
       <c r="N47" s="9" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="O47" s="9" t="s">
         <v>105</v>
       </c>
       <c r="P47" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="Q47" s="8">
         <v>45985</v>
@@ -4646,7 +4646,7 @@
     </row>
     <row r="48" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A48" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B48" s="5">
         <v>46108.75703761574</v>
@@ -4658,16 +4658,16 @@
         <v>46260.58077393519</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F48" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G48" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="H48" s="6" t="s">
         <v>164</v>
-      </c>
-      <c r="H48" s="6" t="s">
-        <v>165</v>
       </c>
       <c r="I48" s="5">
         <v>46202</v>
@@ -4685,13 +4685,13 @@
         <v>26</v>
       </c>
       <c r="N48" s="6" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="O48" s="6" t="s">
         <v>107</v>
       </c>
       <c r="P48" s="6" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="Q48" s="5">
         <v>46007</v>
@@ -4711,7 +4711,7 @@
     </row>
     <row r="49" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A49" s="7" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B49" s="8">
         <v>46108.75704306713</v>
@@ -4723,16 +4723,16 @@
         <v>46220.16760561343</v>
       </c>
       <c r="E49" s="9" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F49" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G49" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="H49" s="9" t="s">
         <v>164</v>
-      </c>
-      <c r="H49" s="9" t="s">
-        <v>165</v>
       </c>
       <c r="I49" s="8">
         <v>46125</v>
@@ -4753,7 +4753,7 @@
         <v>117</v>
       </c>
       <c r="O49" s="9" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="P49" s="9" t="s">
         <v>117</v>
@@ -4776,7 +4776,7 @@
     </row>
     <row r="50" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A50" s="4" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B50" s="5">
         <v>46108.75705032407</v>
@@ -4788,16 +4788,16 @@
         <v>46154.86746811343</v>
       </c>
       <c r="E50" s="6" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F50" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G50" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="H50" s="6" t="s">
         <v>164</v>
-      </c>
-      <c r="H50" s="6" t="s">
-        <v>165</v>
       </c>
       <c r="I50" s="5">
         <v>46125</v>
@@ -4815,13 +4815,13 @@
         <v>26</v>
       </c>
       <c r="N50" s="6" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="O50" s="6" t="s">
         <v>109</v>
       </c>
       <c r="P50" s="6" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="Q50" s="6"/>
       <c r="R50" s="6"/>
@@ -4831,7 +4831,7 @@
     </row>
     <row r="51" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A51" s="7" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B51" s="8">
         <v>46108.75705728009</v>
@@ -4843,16 +4843,16 @@
         <v>46154.8677641088</v>
       </c>
       <c r="E51" s="9" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="F51" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G51" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="H51" s="9" t="s">
         <v>164</v>
-      </c>
-      <c r="H51" s="9" t="s">
-        <v>165</v>
       </c>
       <c r="I51" s="8">
         <v>46135</v>
@@ -4870,13 +4870,13 @@
         <v>26</v>
       </c>
       <c r="N51" s="9" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="O51" s="9" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="P51" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="Q51" s="9"/>
       <c r="R51" s="9"/>
@@ -4886,7 +4886,7 @@
     </row>
     <row r="52" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A52" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B52" s="5">
         <v>46108.757061435186</v>
@@ -4896,16 +4896,16 @@
         <v>46231.17690494213</v>
       </c>
       <c r="E52" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="F52" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G52" s="6" t="s">
         <v>182</v>
       </c>
-      <c r="F52" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G52" s="6" t="s">
+      <c r="H52" s="6" t="s">
         <v>183</v>
-      </c>
-      <c r="H52" s="6" t="s">
-        <v>184</v>
       </c>
       <c r="I52" s="5">
         <v>46195</v>
@@ -4926,7 +4926,7 @@
         <v>117</v>
       </c>
       <c r="O52" s="6" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="P52" s="6" t="s">
         <v>117</v>
@@ -4949,7 +4949,7 @@
     </row>
     <row r="53" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A53" s="7" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B53" s="8">
         <v>46108.75710696759</v>
@@ -4965,10 +4965,10 @@
         <v>26</v>
       </c>
       <c r="G53" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="H53" s="9" t="s">
         <v>183</v>
-      </c>
-      <c r="H53" s="9" t="s">
-        <v>184</v>
       </c>
       <c r="I53" s="8">
         <v>46195</v>
@@ -4986,13 +4986,13 @@
         <v>26</v>
       </c>
       <c r="N53" s="9" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="O53" s="9" t="s">
         <v>112</v>
       </c>
       <c r="P53" s="9" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="Q53" s="9"/>
       <c r="R53" s="9"/>
@@ -5008,7 +5008,7 @@
     </row>
     <row r="54" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A54" s="4" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B54" s="5">
         <v>46108.757112928244</v>
@@ -5018,16 +5018,16 @@
         <v>46260.580782777775</v>
       </c>
       <c r="E54" s="6" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="F54" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G54" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="H54" s="6" t="s">
         <v>183</v>
-      </c>
-      <c r="H54" s="6" t="s">
-        <v>184</v>
       </c>
       <c r="I54" s="5">
         <v>46210</v>
@@ -5045,13 +5045,13 @@
         <v>26</v>
       </c>
       <c r="N54" s="6" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="O54" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="P54" s="6" t="s">
         <v>190</v>
-      </c>
-      <c r="P54" s="6" t="s">
-        <v>191</v>
       </c>
       <c r="Q54" s="6"/>
       <c r="R54" s="6"/>
@@ -5061,7 +5061,7 @@
     </row>
     <row r="55" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A55" s="7" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B55" s="8">
         <v>46111.50860645833</v>
@@ -5073,7 +5073,7 @@
         <v>46182.69406362269</v>
       </c>
       <c r="E55" s="9" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F55" s="9" t="s">
         <v>26</v>
@@ -5103,7 +5103,7 @@
         <v>117</v>
       </c>
       <c r="O55" s="9" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="P55" s="9" t="s">
         <v>26</v>
@@ -5126,7 +5126,7 @@
     </row>
     <row r="56" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A56" s="4" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B56" s="5">
         <v>46111.508755937495</v>
@@ -5138,7 +5138,7 @@
         <v>46182.69350877315</v>
       </c>
       <c r="E56" s="6" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="F56" s="6" t="s">
         <v>26</v>
@@ -5165,13 +5165,13 @@
         <v>26</v>
       </c>
       <c r="N56" s="6" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="O56" s="6" t="s">
         <v>85</v>
       </c>
       <c r="P56" s="6" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="Q56" s="6"/>
       <c r="R56" s="6"/>
@@ -5181,7 +5181,7 @@
     </row>
     <row r="57" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A57" s="7" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B57" s="8">
         <v>46111.508846770834</v>
@@ -5193,7 +5193,7 @@
         <v>46182.69403748843</v>
       </c>
       <c r="E57" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="F57" s="9" t="s">
         <v>26</v>
@@ -5220,13 +5220,13 @@
         <v>26</v>
       </c>
       <c r="N57" s="9" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="O57" s="9" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="P57" s="9" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="Q57" s="9"/>
       <c r="R57" s="9"/>
@@ -5236,7 +5236,7 @@
     </row>
     <row r="58" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A58" s="4" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B58" s="5">
         <v>46108.75711900463</v>
@@ -5246,7 +5246,7 @@
         <v>46217.85709320602</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="F58" s="6" t="s">
         <v>25</v>
@@ -5270,7 +5270,7 @@
         <v>26</v>
       </c>
       <c r="O58" s="6" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="P58" s="6" t="s">
         <v>26</v>
@@ -5285,7 +5285,7 @@
     </row>
     <row r="59" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A59" s="7" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B59" s="8">
         <v>46108.75712325232</v>
@@ -5297,16 +5297,16 @@
         <v>46222.09270599537</v>
       </c>
       <c r="E59" s="9" t="s">
+        <v>204</v>
+      </c>
+      <c r="F59" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G59" s="9" t="s">
         <v>205</v>
       </c>
-      <c r="F59" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="G59" s="9" t="s">
+      <c r="H59" s="9" t="s">
         <v>206</v>
-      </c>
-      <c r="H59" s="9" t="s">
-        <v>207</v>
       </c>
       <c r="I59" s="9"/>
       <c r="J59" s="8">
@@ -5322,13 +5322,13 @@
         <v>26</v>
       </c>
       <c r="N59" s="9" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="O59" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="P59" s="9" t="s">
         <v>208</v>
-      </c>
-      <c r="P59" s="9" t="s">
-        <v>209</v>
       </c>
       <c r="Q59" s="8">
         <v>46121</v>
@@ -5348,7 +5348,7 @@
     </row>
     <row r="60" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A60" s="4" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B60" s="5">
         <v>46114.552579166666</v>
@@ -5360,16 +5360,16 @@
         <v>46211.84604957176</v>
       </c>
       <c r="E60" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="F60" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G60" s="6" t="s">
         <v>211</v>
       </c>
-      <c r="F60" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G60" s="6" t="s">
+      <c r="H60" s="6" t="s">
         <v>212</v>
-      </c>
-      <c r="H60" s="6" t="s">
-        <v>213</v>
       </c>
       <c r="I60" s="5">
         <v>46121</v>
@@ -5387,13 +5387,13 @@
         <v>26</v>
       </c>
       <c r="N60" s="6" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="O60" s="6" t="s">
         <v>77</v>
       </c>
       <c r="P60" s="6" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="Q60" s="6"/>
       <c r="R60" s="6"/>
@@ -5403,7 +5403,7 @@
     </row>
     <row r="61" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A61" s="7" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B61" s="8">
         <v>46114.552773240735</v>
@@ -5415,16 +5415,16 @@
         <v>46211.846055462964</v>
       </c>
       <c r="E61" s="9" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F61" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G61" s="9" t="s">
+        <v>211</v>
+      </c>
+      <c r="H61" s="9" t="s">
         <v>212</v>
-      </c>
-      <c r="H61" s="9" t="s">
-        <v>213</v>
       </c>
       <c r="I61" s="8">
         <v>46121</v>
@@ -5442,13 +5442,13 @@
         <v>26</v>
       </c>
       <c r="N61" s="9" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="O61" s="9" t="s">
         <v>77</v>
       </c>
       <c r="P61" s="9" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="Q61" s="9"/>
       <c r="R61" s="9"/>
@@ -5458,7 +5458,7 @@
     </row>
     <row r="62" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A62" s="4" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B62" s="5">
         <v>46108.75712855324</v>
@@ -5470,16 +5470,16 @@
         <v>46236.273657928235</v>
       </c>
       <c r="E62" s="6" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F62" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G62" s="6" t="s">
+        <v>205</v>
+      </c>
+      <c r="H62" s="6" t="s">
         <v>206</v>
-      </c>
-      <c r="H62" s="6" t="s">
-        <v>207</v>
       </c>
       <c r="I62" s="5">
         <v>46183</v>
@@ -5497,13 +5497,13 @@
         <v>26</v>
       </c>
       <c r="N62" s="6" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="O62" s="6" t="s">
+        <v>219</v>
+      </c>
+      <c r="P62" s="6" t="s">
         <v>220</v>
-      </c>
-      <c r="P62" s="6" t="s">
-        <v>221</v>
       </c>
       <c r="Q62" s="5">
         <v>46183</v>
@@ -5523,7 +5523,7 @@
     </row>
     <row r="63" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A63" s="7" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B63" s="8">
         <v>46114.55286452547</v>
@@ -5535,16 +5535,16 @@
         <v>46217.85704695602</v>
       </c>
       <c r="E63" s="9" t="s">
+        <v>210</v>
+      </c>
+      <c r="F63" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G63" s="9" t="s">
         <v>211</v>
       </c>
-      <c r="F63" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="G63" s="9" t="s">
+      <c r="H63" s="9" t="s">
         <v>212</v>
-      </c>
-      <c r="H63" s="9" t="s">
-        <v>213</v>
       </c>
       <c r="I63" s="8">
         <v>46183</v>
@@ -5562,13 +5562,13 @@
         <v>26</v>
       </c>
       <c r="N63" s="9" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="O63" s="9" t="s">
+        <v>222</v>
+      </c>
+      <c r="P63" s="9" t="s">
         <v>223</v>
-      </c>
-      <c r="P63" s="9" t="s">
-        <v>224</v>
       </c>
       <c r="Q63" s="9"/>
       <c r="R63" s="9"/>
@@ -5578,7 +5578,7 @@
     </row>
     <row r="64" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A64" s="4" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B64" s="5">
         <v>46114.552966620366</v>
@@ -5590,16 +5590,16 @@
         <v>46217.85705476852</v>
       </c>
       <c r="E64" s="6" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F64" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G64" s="6" t="s">
+        <v>211</v>
+      </c>
+      <c r="H64" s="6" t="s">
         <v>212</v>
-      </c>
-      <c r="H64" s="6" t="s">
-        <v>213</v>
       </c>
       <c r="I64" s="5">
         <v>46183</v>
@@ -5617,13 +5617,13 @@
         <v>26</v>
       </c>
       <c r="N64" s="6" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="O64" s="6" t="s">
+        <v>225</v>
+      </c>
+      <c r="P64" s="6" t="s">
         <v>226</v>
-      </c>
-      <c r="P64" s="6" t="s">
-        <v>227</v>
       </c>
       <c r="Q64" s="6"/>
       <c r="R64" s="6"/>
@@ -5633,7 +5633,7 @@
     </row>
     <row r="65" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A65" s="7" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B65" s="8">
         <v>46108.75713383102</v>
@@ -5651,10 +5651,10 @@
         <v>26</v>
       </c>
       <c r="G65" s="9" t="s">
+        <v>211</v>
+      </c>
+      <c r="H65" s="9" t="s">
         <v>212</v>
-      </c>
-      <c r="H65" s="9" t="s">
-        <v>213</v>
       </c>
       <c r="I65" s="8">
         <v>46190</v>
@@ -5672,13 +5672,13 @@
         <v>26</v>
       </c>
       <c r="N65" s="9" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="O65" s="9" t="s">
+        <v>228</v>
+      </c>
+      <c r="P65" s="9" t="s">
         <v>229</v>
-      </c>
-      <c r="P65" s="9" t="s">
-        <v>230</v>
       </c>
       <c r="Q65" s="8">
         <v>46190</v>
@@ -5698,7 +5698,7 @@
     </row>
     <row r="66" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A66" s="4" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B66" s="5">
         <v>46114.55312298611</v>
@@ -5708,16 +5708,16 @@
         <v>46217.85705168982</v>
       </c>
       <c r="E66" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="F66" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G66" s="6" t="s">
         <v>211</v>
       </c>
-      <c r="F66" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G66" s="6" t="s">
+      <c r="H66" s="6" t="s">
         <v>212</v>
-      </c>
-      <c r="H66" s="6" t="s">
-        <v>213</v>
       </c>
       <c r="I66" s="6"/>
       <c r="J66" s="5">
@@ -5736,7 +5736,7 @@
         <v>106</v>
       </c>
       <c r="O66" s="6" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="P66" s="6" t="s">
         <v>26</v>
@@ -5749,7 +5749,7 @@
     </row>
     <row r="67" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A67" s="7" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B67" s="8">
         <v>46114.553244675924</v>
@@ -5759,16 +5759,16 @@
         <v>46217.85706487269</v>
       </c>
       <c r="E67" s="9" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="F67" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G67" s="9" t="s">
+        <v>211</v>
+      </c>
+      <c r="H67" s="9" t="s">
         <v>212</v>
-      </c>
-      <c r="H67" s="9" t="s">
-        <v>213</v>
       </c>
       <c r="I67" s="9"/>
       <c r="J67" s="8">
@@ -5787,7 +5787,7 @@
         <v>106</v>
       </c>
       <c r="O67" s="9" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="P67" s="9" t="s">
         <v>26</v>
@@ -5800,7 +5800,7 @@
     </row>
     <row r="68" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A68" s="4" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B68" s="5">
         <v>46108.757138761575</v>
@@ -5810,16 +5810,16 @@
         <v>46114.631384050925</v>
       </c>
       <c r="E68" s="6" t="s">
+        <v>234</v>
+      </c>
+      <c r="F68" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G68" s="6" t="s">
         <v>235</v>
       </c>
-      <c r="F68" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G68" s="6" t="s">
+      <c r="H68" s="6" t="s">
         <v>236</v>
-      </c>
-      <c r="H68" s="6" t="s">
-        <v>237</v>
       </c>
       <c r="I68" s="5">
         <v>46281</v>
@@ -5837,10 +5837,10 @@
         <v>26</v>
       </c>
       <c r="N68" s="6" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="O68" s="6" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="P68" s="6" t="s">
         <v>26</v>
@@ -5863,7 +5863,7 @@
     </row>
     <row r="69" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A69" s="7" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B69" s="8">
         <v>46111.55280189815</v>
@@ -5873,16 +5873,16 @@
         <v>46114.62851033565</v>
       </c>
       <c r="E69" s="9" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F69" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G69" s="9" t="s">
+        <v>235</v>
+      </c>
+      <c r="H69" s="9" t="s">
         <v>236</v>
-      </c>
-      <c r="H69" s="9" t="s">
-        <v>237</v>
       </c>
       <c r="I69" s="9"/>
       <c r="J69" s="8">
@@ -5898,13 +5898,13 @@
         <v>26</v>
       </c>
       <c r="N69" s="9" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="O69" s="9" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="P69" s="9" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="Q69" s="9"/>
       <c r="R69" s="9"/>
@@ -5914,7 +5914,7 @@
     </row>
     <row r="70" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A70" s="4" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B70" s="5">
         <v>46111.55285245371</v>
@@ -5924,16 +5924,16 @@
         <v>46114.62851040509</v>
       </c>
       <c r="E70" s="6" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="F70" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G70" s="6" t="s">
+        <v>235</v>
+      </c>
+      <c r="H70" s="6" t="s">
         <v>236</v>
-      </c>
-      <c r="H70" s="6" t="s">
-        <v>237</v>
       </c>
       <c r="I70" s="6"/>
       <c r="J70" s="5">
@@ -5949,13 +5949,13 @@
         <v>26</v>
       </c>
       <c r="N70" s="6" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="O70" s="6" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="P70" s="6" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="Q70" s="6"/>
       <c r="R70" s="6"/>
@@ -5965,7 +5965,7 @@
     </row>
     <row r="71" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A71" s="7" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B71" s="8">
         <v>46108.75714166666</v>
@@ -5975,7 +5975,7 @@
         <v>46118.545566597226</v>
       </c>
       <c r="E71" s="9" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F71" s="9" t="s">
         <v>25</v>
@@ -5999,7 +5999,7 @@
         <v>26</v>
       </c>
       <c r="O71" s="9" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="P71" s="9" t="s">
         <v>26</v>
@@ -6012,7 +6012,7 @@
     </row>
     <row r="72" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A72" s="4" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B72" s="5">
         <v>46108.75714454861</v>
@@ -6022,16 +6022,16 @@
         <v>46240.16751462963</v>
       </c>
       <c r="E72" s="6" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="F72" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G72" s="6" t="s">
+        <v>247</v>
+      </c>
+      <c r="H72" s="6" t="s">
         <v>248</v>
-      </c>
-      <c r="H72" s="6" t="s">
-        <v>249</v>
       </c>
       <c r="I72" s="6"/>
       <c r="J72" s="5">
@@ -6047,13 +6047,13 @@
         <v>26</v>
       </c>
       <c r="N72" s="6" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="O72" s="6" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="P72" s="6" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="Q72" s="5">
         <v>46231</v>
@@ -6073,7 +6073,7 @@
     </row>
     <row r="73" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A73" s="7" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B73" s="8">
         <v>46111.50359008102</v>
@@ -6085,7 +6085,7 @@
         <v>46260.58097469907</v>
       </c>
       <c r="E73" s="9" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="F73" s="9" t="s">
         <v>25</v>
@@ -6109,7 +6109,7 @@
         <v>26</v>
       </c>
       <c r="O73" s="9" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="P73" s="9" t="s">
         <v>26</v>
@@ -6126,7 +6126,7 @@
     </row>
     <row r="74" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A74" s="4" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B74" s="5">
         <v>46111.50404616898</v>
@@ -6138,16 +6138,16 @@
         <v>46260.58079141204</v>
       </c>
       <c r="E74" s="6" t="s">
+        <v>254</v>
+      </c>
+      <c r="F74" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G74" s="6" t="s">
         <v>255</v>
       </c>
-      <c r="F74" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G74" s="6" t="s">
+      <c r="H74" s="6" t="s">
         <v>256</v>
-      </c>
-      <c r="H74" s="6" t="s">
-        <v>257</v>
       </c>
       <c r="I74" s="5">
         <v>46211</v>
@@ -6165,13 +6165,13 @@
         <v>26</v>
       </c>
       <c r="N74" s="6" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="O74" s="6" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="P74" s="6" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="Q74" s="5">
         <v>46211</v>
@@ -6191,7 +6191,7 @@
     </row>
     <row r="75" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A75" s="7" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B75" s="8">
         <v>46111.50406170139</v>
@@ -6203,16 +6203,16 @@
         <v>46260.580961342595</v>
       </c>
       <c r="E75" s="9" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="F75" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G75" s="9" t="s">
+        <v>247</v>
+      </c>
+      <c r="H75" s="9" t="s">
         <v>248</v>
-      </c>
-      <c r="H75" s="9" t="s">
-        <v>249</v>
       </c>
       <c r="I75" s="8">
         <v>46213</v>
@@ -6230,13 +6230,13 @@
         <v>26</v>
       </c>
       <c r="N75" s="9" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="O75" s="9" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="P75" s="9" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="Q75" s="8">
         <v>46213</v>
@@ -6256,7 +6256,7 @@
     </row>
     <row r="76" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A76" s="4" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B76" s="5">
         <v>46111.50543856481</v>
@@ -6266,7 +6266,7 @@
         <v>46260.577887962965</v>
       </c>
       <c r="E76" s="6" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="F76" s="6" t="s">
         <v>25</v>
@@ -6290,7 +6290,7 @@
         <v>26</v>
       </c>
       <c r="O76" s="6" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="P76" s="6" t="s">
         <v>26</v>
@@ -6305,7 +6305,7 @@
     </row>
     <row r="77" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A77" s="7" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B77" s="8">
         <v>46111.505495046295</v>
@@ -6317,16 +6317,16 @@
         <v>46260.58096115741</v>
       </c>
       <c r="E77" s="9" t="s">
+        <v>265</v>
+      </c>
+      <c r="F77" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G77" s="9" t="s">
         <v>266</v>
       </c>
-      <c r="F77" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="G77" s="9" t="s">
+      <c r="H77" s="9" t="s">
         <v>267</v>
-      </c>
-      <c r="H77" s="9" t="s">
-        <v>268</v>
       </c>
       <c r="I77" s="8">
         <v>46217</v>
@@ -6344,13 +6344,13 @@
         <v>26</v>
       </c>
       <c r="N77" s="9" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="O77" s="9" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="P77" s="9" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="Q77" s="8">
         <v>46217</v>
@@ -6370,7 +6370,7 @@
     </row>
     <row r="78" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A78" s="4" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B78" s="5">
         <v>46111.50560314815</v>
@@ -6382,16 +6382,16 @@
         <v>46260.57750302083</v>
       </c>
       <c r="E78" s="6" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="F78" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G78" s="6" t="s">
+        <v>266</v>
+      </c>
+      <c r="H78" s="6" t="s">
         <v>267</v>
-      </c>
-      <c r="H78" s="6" t="s">
-        <v>268</v>
       </c>
       <c r="I78" s="5">
         <v>46226</v>
@@ -6409,13 +6409,13 @@
         <v>26</v>
       </c>
       <c r="N78" s="6" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="O78" s="6" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="P78" s="6" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="Q78" s="5">
         <v>46226</v>
@@ -6435,7 +6435,7 @@
     </row>
     <row r="79" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A79" s="7" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B79" s="8">
         <v>46111.52633317129</v>
@@ -6447,16 +6447,16 @@
         <v>46260.57746712963</v>
       </c>
       <c r="E79" s="9" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F79" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G79" s="9" t="s">
+        <v>266</v>
+      </c>
+      <c r="H79" s="9" t="s">
         <v>267</v>
-      </c>
-      <c r="H79" s="9" t="s">
-        <v>268</v>
       </c>
       <c r="I79" s="8">
         <v>46226</v>
@@ -6474,13 +6474,13 @@
         <v>26</v>
       </c>
       <c r="N79" s="9" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="O79" s="9" t="s">
+        <v>273</v>
+      </c>
+      <c r="P79" s="9" t="s">
         <v>274</v>
-      </c>
-      <c r="P79" s="9" t="s">
-        <v>275</v>
       </c>
       <c r="Q79" s="9"/>
       <c r="R79" s="9"/>
@@ -6490,7 +6490,7 @@
     </row>
     <row r="80" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A80" s="4" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B80" s="5">
         <v>46111.526644375</v>
@@ -6502,16 +6502,16 @@
         <v>46260.57747775463</v>
       </c>
       <c r="E80" s="6" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F80" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G80" s="6" t="s">
+        <v>266</v>
+      </c>
+      <c r="H80" s="6" t="s">
         <v>267</v>
-      </c>
-      <c r="H80" s="6" t="s">
-        <v>268</v>
       </c>
       <c r="I80" s="5">
         <v>46226</v>
@@ -6529,13 +6529,13 @@
         <v>26</v>
       </c>
       <c r="N80" s="6" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="O80" s="6" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="P80" s="6" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="Q80" s="6"/>
       <c r="R80" s="6"/>
@@ -6545,7 +6545,7 @@
     </row>
     <row r="81" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A81" s="7" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B81" s="8">
         <v>46111.50563458333</v>
@@ -6557,16 +6557,16 @@
         <v>46260.57788128473</v>
       </c>
       <c r="E81" s="9" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F81" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G81" s="9" t="s">
+        <v>247</v>
+      </c>
+      <c r="H81" s="9" t="s">
         <v>248</v>
-      </c>
-      <c r="H81" s="9" t="s">
-        <v>249</v>
       </c>
       <c r="I81" s="8">
         <v>46246</v>
@@ -6584,13 +6584,13 @@
         <v>26</v>
       </c>
       <c r="N81" s="9" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="O81" s="9" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="P81" s="9" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="Q81" s="8">
         <v>46246</v>
@@ -6610,7 +6610,7 @@
     </row>
     <row r="82" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A82" s="4" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B82" s="5">
         <v>46111.526916469906</v>
@@ -6622,16 +6622,16 @@
         <v>46260.57783230324</v>
       </c>
       <c r="E82" s="6" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F82" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G82" s="6" t="s">
+        <v>247</v>
+      </c>
+      <c r="H82" s="6" t="s">
         <v>248</v>
-      </c>
-      <c r="H82" s="6" t="s">
-        <v>249</v>
       </c>
       <c r="I82" s="5">
         <v>46246</v>
@@ -6649,13 +6649,13 @@
         <v>26</v>
       </c>
       <c r="N82" s="6" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="O82" s="6" t="s">
+        <v>280</v>
+      </c>
+      <c r="P82" s="6" t="s">
         <v>281</v>
-      </c>
-      <c r="P82" s="6" t="s">
-        <v>282</v>
       </c>
       <c r="Q82" s="6"/>
       <c r="R82" s="6"/>
@@ -6665,7 +6665,7 @@
     </row>
     <row r="83" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A83" s="7" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B83" s="8">
         <v>46111.52699828704</v>
@@ -6677,16 +6677,16 @@
         <v>46260.57784520833</v>
       </c>
       <c r="E83" s="9" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F83" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G83" s="9" t="s">
+        <v>247</v>
+      </c>
+      <c r="H83" s="9" t="s">
         <v>248</v>
-      </c>
-      <c r="H83" s="9" t="s">
-        <v>249</v>
       </c>
       <c r="I83" s="8">
         <v>46246</v>
@@ -6704,13 +6704,13 @@
         <v>26</v>
       </c>
       <c r="N83" s="9" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="O83" s="9" t="s">
+        <v>283</v>
+      </c>
+      <c r="P83" s="9" t="s">
         <v>284</v>
-      </c>
-      <c r="P83" s="9" t="s">
-        <v>285</v>
       </c>
       <c r="Q83" s="9"/>
       <c r="R83" s="9"/>
@@ -6720,7 +6720,7 @@
     </row>
     <row r="84" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A84" s="4" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B84" s="5">
         <v>46108.75714884259</v>
@@ -6730,7 +6730,7 @@
         <v>46221.1155655787</v>
       </c>
       <c r="E84" s="6" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="F84" s="6" t="s">
         <v>25</v>
@@ -6754,7 +6754,7 @@
         <v>26</v>
       </c>
       <c r="O84" s="6" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="P84" s="6" t="s">
         <v>26</v>
@@ -6767,7 +6767,7 @@
     </row>
     <row r="85" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A85" s="7" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B85" s="8">
         <v>46108.75715243055</v>
@@ -6777,16 +6777,16 @@
         <v>46185.184959907405</v>
       </c>
       <c r="E85" s="9" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="F85" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G85" s="9" t="s">
+        <v>255</v>
+      </c>
+      <c r="H85" s="9" t="s">
         <v>256</v>
-      </c>
-      <c r="H85" s="9" t="s">
-        <v>257</v>
       </c>
       <c r="I85" s="8">
         <v>46183</v>
@@ -6804,13 +6804,13 @@
         <v>26</v>
       </c>
       <c r="N85" s="9" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="O85" s="9" t="s">
         <v>147</v>
       </c>
       <c r="P85" s="9" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="Q85" s="8">
         <v>46183</v>
@@ -6830,7 +6830,7 @@
     </row>
     <row r="86" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A86" s="4" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B86" s="5">
         <v>46108.75715773148</v>
@@ -6846,10 +6846,10 @@
         <v>26</v>
       </c>
       <c r="G86" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="H86" s="6" t="s">
         <v>256</v>
-      </c>
-      <c r="H86" s="6" t="s">
-        <v>257</v>
       </c>
       <c r="I86" s="5">
         <v>46239</v>
@@ -6867,13 +6867,13 @@
         <v>26</v>
       </c>
       <c r="N86" s="6" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="O86" s="6" t="s">
         <v>138</v>
       </c>
       <c r="P86" s="6" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="Q86" s="5">
         <v>46239</v>
@@ -6893,7 +6893,7 @@
     </row>
     <row r="87" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A87" s="7" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B87" s="8">
         <v>46108.75716349537</v>
@@ -6903,16 +6903,16 @@
         <v>46248.16971915509</v>
       </c>
       <c r="E87" s="9" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F87" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G87" s="9" t="s">
+        <v>255</v>
+      </c>
+      <c r="H87" s="9" t="s">
         <v>256</v>
-      </c>
-      <c r="H87" s="9" t="s">
-        <v>257</v>
       </c>
       <c r="I87" s="8">
         <v>46246</v>
@@ -6930,13 +6930,13 @@
         <v>26</v>
       </c>
       <c r="N87" s="9" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="O87" s="9" t="s">
         <v>129</v>
       </c>
       <c r="P87" s="9" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="Q87" s="8">
         <v>46246</v>
@@ -6956,7 +6956,7 @@
     </row>
     <row r="88" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A88" s="4" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B88" s="5">
         <v>46108.75716875</v>
@@ -6966,16 +6966,16 @@
         <v>46267.17843465278</v>
       </c>
       <c r="E88" s="6" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="F88" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G88" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="H88" s="6" t="s">
         <v>256</v>
-      </c>
-      <c r="H88" s="6" t="s">
-        <v>257</v>
       </c>
       <c r="I88" s="5">
         <v>46273</v>
@@ -6993,13 +6993,13 @@
         <v>26</v>
       </c>
       <c r="N88" s="6" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="O88" s="6" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="P88" s="6" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="Q88" s="5">
         <v>46273</v>
@@ -7011,7 +7011,7 @@
         <v>0</v>
       </c>
       <c r="T88" s="12" t="s">
-        <v>152</v>
+        <v>298</v>
       </c>
       <c r="U88" s="10" t="s">
         <v>53</v>
@@ -7035,10 +7035,10 @@
         <v>26</v>
       </c>
       <c r="G89" s="9" t="s">
+        <v>255</v>
+      </c>
+      <c r="H89" s="9" t="s">
         <v>256</v>
-      </c>
-      <c r="H89" s="9" t="s">
-        <v>257</v>
       </c>
       <c r="I89" s="8">
         <v>46220</v>
@@ -7056,13 +7056,13 @@
         <v>26</v>
       </c>
       <c r="N89" s="9" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="O89" s="9" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="P89" s="9" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="Q89" s="8">
         <v>46220</v>
@@ -7098,10 +7098,10 @@
         <v>26</v>
       </c>
       <c r="G90" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="H90" s="6" t="s">
         <v>256</v>
-      </c>
-      <c r="H90" s="6" t="s">
-        <v>257</v>
       </c>
       <c r="I90" s="6"/>
       <c r="J90" s="5">
@@ -7117,10 +7117,10 @@
         <v>26</v>
       </c>
       <c r="N90" s="6" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="O90" s="6" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="P90" s="6" t="s">
         <v>303</v>
@@ -7159,10 +7159,10 @@
         <v>26</v>
       </c>
       <c r="G91" s="9" t="s">
+        <v>255</v>
+      </c>
+      <c r="H91" s="9" t="s">
         <v>256</v>
-      </c>
-      <c r="H91" s="9" t="s">
-        <v>257</v>
       </c>
       <c r="I91" s="8">
         <v>46181</v>
@@ -7180,10 +7180,10 @@
         <v>26</v>
       </c>
       <c r="N91" s="9" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="O91" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="P91" s="9" t="s">
         <v>306</v>
@@ -7293,7 +7293,7 @@
         <v>308</v>
       </c>
       <c r="O93" s="9" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="P93" s="9" t="s">
         <v>308</v>
@@ -7326,7 +7326,7 @@
         <v>46267.167487708335</v>
       </c>
       <c r="E94" s="6" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F94" s="6" t="s">
         <v>26</v>
@@ -7379,7 +7379,7 @@
         <v>46267.167488796294</v>
       </c>
       <c r="E95" s="9" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F95" s="9" t="s">
         <v>26</v>
@@ -7462,7 +7462,7 @@
         <v>308</v>
       </c>
       <c r="O96" s="6" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="P96" s="6" t="s">
         <v>308</v>
@@ -7495,7 +7495,7 @@
         <v>46269.167690648144</v>
       </c>
       <c r="E97" s="9" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F97" s="9" t="s">
         <v>26</v>
@@ -7548,7 +7548,7 @@
         <v>46269.16769188657</v>
       </c>
       <c r="E98" s="6" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F98" s="6" t="s">
         <v>26</v>
@@ -7598,7 +7598,7 @@
       </c>
       <c r="C99" s="9"/>
       <c r="D99" s="8">
-        <v>46266.176813287035</v>
+        <v>46273.16745574074</v>
       </c>
       <c r="E99" s="9" t="s">
         <v>327</v>
@@ -7631,7 +7631,7 @@
         <v>308</v>
       </c>
       <c r="O99" s="9" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="P99" s="9" t="s">
         <v>308</v>
@@ -7646,7 +7646,7 @@
         <v>0</v>
       </c>
       <c r="T99" s="12" t="s">
-        <v>152</v>
+        <v>298</v>
       </c>
       <c r="U99" s="10" t="s">
         <v>53</v>
@@ -7661,10 +7661,10 @@
       </c>
       <c r="C100" s="6"/>
       <c r="D100" s="5">
-        <v>46227.72251393519</v>
+        <v>46273.16745900463</v>
       </c>
       <c r="E100" s="6" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F100" s="6" t="s">
         <v>26</v>
@@ -7714,10 +7714,10 @@
       </c>
       <c r="C101" s="9"/>
       <c r="D101" s="8">
-        <v>46227.72251137732</v>
+        <v>46273.16746020834</v>
       </c>
       <c r="E101" s="9" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F101" s="9" t="s">
         <v>26</v>
@@ -7800,7 +7800,7 @@
         <v>308</v>
       </c>
       <c r="O102" s="6" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="P102" s="6" t="s">
         <v>308</v>
@@ -7815,7 +7815,7 @@
         <v>0</v>
       </c>
       <c r="T102" s="12" t="s">
-        <v>152</v>
+        <v>298</v>
       </c>
       <c r="U102" s="10" t="s">
         <v>53</v>
@@ -7833,7 +7833,7 @@
         <v>46227.722512928245</v>
       </c>
       <c r="E103" s="9" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F103" s="9" t="s">
         <v>26</v>
@@ -7886,7 +7886,7 @@
         <v>46227.72251365741</v>
       </c>
       <c r="E104" s="6" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F104" s="6" t="s">
         <v>26</v>
@@ -7969,7 +7969,7 @@
         <v>308</v>
       </c>
       <c r="O105" s="9" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="P105" s="9" t="s">
         <v>308</v>
@@ -7984,7 +7984,7 @@
         <v>0</v>
       </c>
       <c r="T105" s="12" t="s">
-        <v>152</v>
+        <v>298</v>
       </c>
       <c r="U105" s="10" t="s">
         <v>53</v>
@@ -8002,7 +8002,7 @@
         <v>46227.722511921296</v>
       </c>
       <c r="E106" s="6" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F106" s="6" t="s">
         <v>26</v>
@@ -8055,7 +8055,7 @@
         <v>46227.72251247685</v>
       </c>
       <c r="E107" s="9" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F107" s="9" t="s">
         <v>26</v>
@@ -8105,7 +8105,7 @@
       </c>
       <c r="C108" s="6"/>
       <c r="D108" s="5">
-        <v>46245.73985467592</v>
+        <v>46273.13886990741</v>
       </c>
       <c r="E108" s="6" t="s">
         <v>349</v>
@@ -8138,7 +8138,7 @@
         <v>308</v>
       </c>
       <c r="O108" s="6" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="P108" s="6" t="s">
         <v>308</v>
@@ -8152,8 +8152,8 @@
       <c r="S108" s="6">
         <v>0</v>
       </c>
-      <c r="T108" s="11" t="s">
-        <v>127</v>
+      <c r="T108" s="12" t="s">
+        <v>298</v>
       </c>
       <c r="U108" s="10" t="s">
         <v>53</v>
@@ -8171,7 +8171,7 @@
         <v>46223.59502533565</v>
       </c>
       <c r="E109" s="9" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F109" s="9" t="s">
         <v>26</v>
@@ -8199,7 +8199,7 @@
         <v>349</v>
       </c>
       <c r="O109" s="9" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="P109" s="9" t="s">
         <v>351</v>
@@ -8222,7 +8222,7 @@
         <v>46223.59502458334</v>
       </c>
       <c r="E110" s="6" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F110" s="6" t="s">
         <v>26</v>
@@ -8250,7 +8250,7 @@
         <v>349</v>
       </c>
       <c r="O110" s="6" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="P110" s="6" t="s">
         <v>353</v>
@@ -8334,7 +8334,7 @@
         <v>46223.595106875</v>
       </c>
       <c r="E112" s="6" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F112" s="6" t="s">
         <v>26</v>
@@ -8362,7 +8362,7 @@
         <v>355</v>
       </c>
       <c r="O112" s="6" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="P112" s="6" t="s">
         <v>358</v>
@@ -8385,7 +8385,7 @@
         <v>46223.59510622685</v>
       </c>
       <c r="E113" s="9" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F113" s="9" t="s">
         <v>26</v>
@@ -8413,7 +8413,7 @@
         <v>355</v>
       </c>
       <c r="O113" s="9" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="P113" s="9" t="s">
         <v>360</v>
@@ -8546,7 +8546,7 @@
         <v>46114.62888387732</v>
       </c>
       <c r="E116" s="6" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F116" s="6" t="s">
         <v>26</v>
@@ -8574,7 +8574,7 @@
         <v>365</v>
       </c>
       <c r="O116" s="6" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="P116" s="6" t="s">
         <v>370</v>
@@ -8597,7 +8597,7 @@
         <v>46114.62888469908</v>
       </c>
       <c r="E117" s="9" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F117" s="9" t="s">
         <v>26</v>
@@ -8625,7 +8625,7 @@
         <v>365</v>
       </c>
       <c r="O117" s="9" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="P117" s="9" t="s">
         <v>372</v>
@@ -8966,7 +8966,7 @@
         <v>46223.595359328705</v>
       </c>
       <c r="E124" s="6" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F124" s="6" t="s">
         <v>26</v>
@@ -8996,7 +8996,7 @@
         <v>385</v>
       </c>
       <c r="O124" s="6" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="P124" s="6" t="s">
         <v>388</v>
@@ -9019,7 +9019,7 @@
         <v>46223.59535869213</v>
       </c>
       <c r="E125" s="9" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F125" s="9" t="s">
         <v>26</v>
@@ -9049,7 +9049,7 @@
         <v>385</v>
       </c>
       <c r="O125" s="9" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="P125" s="9" t="s">
         <v>390</v>
@@ -9343,10 +9343,10 @@
         <v>26</v>
       </c>
       <c r="G131" s="9" t="s">
+        <v>266</v>
+      </c>
+      <c r="H131" s="9" t="s">
         <v>267</v>
-      </c>
-      <c r="H131" s="9" t="s">
-        <v>268</v>
       </c>
       <c r="I131" s="8">
         <v>46293</v>
@@ -9400,16 +9400,16 @@
         <v>46114.62931347222</v>
       </c>
       <c r="E132" s="6" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F132" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G132" s="6" t="s">
+        <v>266</v>
+      </c>
+      <c r="H132" s="6" t="s">
         <v>267</v>
-      </c>
-      <c r="H132" s="6" t="s">
-        <v>268</v>
       </c>
       <c r="I132" s="6"/>
       <c r="J132" s="5">
@@ -9428,7 +9428,7 @@
         <v>402</v>
       </c>
       <c r="O132" s="6" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="P132" s="6" t="s">
         <v>405</v>
@@ -9451,16 +9451,16 @@
         <v>46114.62931429398</v>
       </c>
       <c r="E133" s="9" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F133" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G133" s="9" t="s">
+        <v>266</v>
+      </c>
+      <c r="H133" s="9" t="s">
         <v>267</v>
-      </c>
-      <c r="H133" s="9" t="s">
-        <v>268</v>
       </c>
       <c r="I133" s="9"/>
       <c r="J133" s="8">
@@ -9479,7 +9479,7 @@
         <v>402</v>
       </c>
       <c r="O133" s="9" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="P133" s="9" t="s">
         <v>407</v>
@@ -9508,10 +9508,10 @@
         <v>26</v>
       </c>
       <c r="G134" s="6" t="s">
+        <v>266</v>
+      </c>
+      <c r="H134" s="6" t="s">
         <v>267</v>
-      </c>
-      <c r="H134" s="6" t="s">
-        <v>268</v>
       </c>
       <c r="I134" s="6"/>
       <c r="J134" s="5">
@@ -9559,10 +9559,10 @@
         <v>26</v>
       </c>
       <c r="G135" s="9" t="s">
+        <v>266</v>
+      </c>
+      <c r="H135" s="9" t="s">
         <v>267</v>
-      </c>
-      <c r="H135" s="9" t="s">
-        <v>268</v>
       </c>
       <c r="I135" s="9"/>
       <c r="J135" s="8">
@@ -9610,10 +9610,10 @@
         <v>26</v>
       </c>
       <c r="G136" s="6" t="s">
+        <v>266</v>
+      </c>
+      <c r="H136" s="6" t="s">
         <v>267</v>
-      </c>
-      <c r="H136" s="6" t="s">
-        <v>268</v>
       </c>
       <c r="I136" s="6"/>
       <c r="J136" s="5">
@@ -9661,10 +9661,10 @@
         <v>26</v>
       </c>
       <c r="G137" s="9" t="s">
+        <v>266</v>
+      </c>
+      <c r="H137" s="9" t="s">
         <v>267</v>
-      </c>
-      <c r="H137" s="9" t="s">
-        <v>268</v>
       </c>
       <c r="I137" s="9"/>
       <c r="J137" s="8">
@@ -9712,10 +9712,10 @@
         <v>26</v>
       </c>
       <c r="G138" s="6" t="s">
+        <v>266</v>
+      </c>
+      <c r="H138" s="6" t="s">
         <v>267</v>
-      </c>
-      <c r="H138" s="6" t="s">
-        <v>268</v>
       </c>
       <c r="I138" s="6"/>
       <c r="J138" s="5">
@@ -9763,10 +9763,10 @@
         <v>26</v>
       </c>
       <c r="G139" s="9" t="s">
+        <v>266</v>
+      </c>
+      <c r="H139" s="9" t="s">
         <v>267</v>
-      </c>
-      <c r="H139" s="9" t="s">
-        <v>268</v>
       </c>
       <c r="I139" s="8">
         <v>46294</v>
@@ -9820,16 +9820,16 @@
         <v>46114.830281076385</v>
       </c>
       <c r="E140" s="6" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F140" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G140" s="6" t="s">
+        <v>266</v>
+      </c>
+      <c r="H140" s="6" t="s">
         <v>267</v>
-      </c>
-      <c r="H140" s="6" t="s">
-        <v>268</v>
       </c>
       <c r="I140" s="5">
         <v>46294</v>
@@ -9850,7 +9850,7 @@
         <v>420</v>
       </c>
       <c r="O140" s="6" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="P140" s="6" t="s">
         <v>423</v>
@@ -9873,16 +9873,16 @@
         <v>46114.830302789356</v>
       </c>
       <c r="E141" s="9" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F141" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G141" s="9" t="s">
+        <v>266</v>
+      </c>
+      <c r="H141" s="9" t="s">
         <v>267</v>
-      </c>
-      <c r="H141" s="9" t="s">
-        <v>268</v>
       </c>
       <c r="I141" s="8">
         <v>46294</v>
@@ -9903,7 +9903,7 @@
         <v>420</v>
       </c>
       <c r="O141" s="9" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="P141" s="9" t="s">
         <v>420</v>
@@ -9932,10 +9932,10 @@
         <v>26</v>
       </c>
       <c r="G142" s="6" t="s">
+        <v>266</v>
+      </c>
+      <c r="H142" s="6" t="s">
         <v>267</v>
-      </c>
-      <c r="H142" s="6" t="s">
-        <v>268</v>
       </c>
       <c r="I142" s="5">
         <v>46294</v>
@@ -9985,10 +9985,10 @@
         <v>26</v>
       </c>
       <c r="G143" s="9" t="s">
+        <v>266</v>
+      </c>
+      <c r="H143" s="9" t="s">
         <v>267</v>
-      </c>
-      <c r="H143" s="9" t="s">
-        <v>268</v>
       </c>
       <c r="I143" s="8">
         <v>46294</v>
@@ -10038,10 +10038,10 @@
         <v>26</v>
       </c>
       <c r="G144" s="6" t="s">
+        <v>266</v>
+      </c>
+      <c r="H144" s="6" t="s">
         <v>267</v>
-      </c>
-      <c r="H144" s="6" t="s">
-        <v>268</v>
       </c>
       <c r="I144" s="5">
         <v>46294</v>
@@ -10091,10 +10091,10 @@
         <v>26</v>
       </c>
       <c r="G145" s="9" t="s">
+        <v>266</v>
+      </c>
+      <c r="H145" s="9" t="s">
         <v>267</v>
-      </c>
-      <c r="H145" s="9" t="s">
-        <v>268</v>
       </c>
       <c r="I145" s="8">
         <v>46294</v>
@@ -10144,10 +10144,10 @@
         <v>26</v>
       </c>
       <c r="G146" s="6" t="s">
+        <v>266</v>
+      </c>
+      <c r="H146" s="6" t="s">
         <v>267</v>
-      </c>
-      <c r="H146" s="6" t="s">
-        <v>268</v>
       </c>
       <c r="I146" s="5">
         <v>46294</v>

</xml_diff>

<commit_message>
Actualizacion automatica 2026-09-09 17:12 UTC
</commit_message>
<xml_diff>
--- a/data/50001525 - ZITRON PERU METRO LIMA E07.xlsx
+++ b/data/50001525 - ZITRON PERU METRO LIMA E07.xlsx
@@ -727,6 +727,9 @@
     <t>OT 4287 ZVR 1-14-42/4,OT  4288 ZVR1-14-30/4</t>
   </si>
   <si>
+    <t>Media</t>
+  </si>
+  <si>
     <t>1213869987281952</t>
   </si>
   <si>
@@ -905,9 +908,6 @@
   </si>
   <si>
     <t>Recepcion motor</t>
-  </si>
-  <si>
-    <t>Media</t>
   </si>
   <si>
     <t>1213833564713244</t>
@@ -5807,7 +5807,7 @@
       </c>
       <c r="C68" s="6"/>
       <c r="D68" s="5">
-        <v>46114.631384050925</v>
+        <v>46274.137942905094</v>
       </c>
       <c r="E68" s="6" t="s">
         <v>234</v>
@@ -5854,8 +5854,8 @@
       <c r="S68" s="6">
         <v>0</v>
       </c>
-      <c r="T68" s="11" t="s">
-        <v>127</v>
+      <c r="T68" s="12" t="s">
+        <v>238</v>
       </c>
       <c r="U68" s="10" t="s">
         <v>53</v>
@@ -5863,7 +5863,7 @@
     </row>
     <row r="69" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A69" s="7" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B69" s="8">
         <v>46111.55280189815</v>
@@ -5904,7 +5904,7 @@
         <v>210</v>
       </c>
       <c r="P69" s="9" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="Q69" s="9"/>
       <c r="R69" s="9"/>
@@ -5914,7 +5914,7 @@
     </row>
     <row r="70" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A70" s="4" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B70" s="5">
         <v>46111.55285245371</v>
@@ -5924,7 +5924,7 @@
         <v>46114.62851040509</v>
       </c>
       <c r="E70" s="6" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="F70" s="6" t="s">
         <v>26</v>
@@ -5955,7 +5955,7 @@
         <v>215</v>
       </c>
       <c r="P70" s="6" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="Q70" s="6"/>
       <c r="R70" s="6"/>
@@ -5965,7 +5965,7 @@
     </row>
     <row r="71" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A71" s="7" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B71" s="8">
         <v>46108.75714166666</v>
@@ -5975,7 +5975,7 @@
         <v>46118.545566597226</v>
       </c>
       <c r="E71" s="9" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="F71" s="9" t="s">
         <v>25</v>
@@ -5999,7 +5999,7 @@
         <v>26</v>
       </c>
       <c r="O71" s="9" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="P71" s="9" t="s">
         <v>26</v>
@@ -6012,7 +6012,7 @@
     </row>
     <row r="72" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A72" s="4" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B72" s="5">
         <v>46108.75714454861</v>
@@ -6022,16 +6022,16 @@
         <v>46240.16751462963</v>
       </c>
       <c r="E72" s="6" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="F72" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G72" s="6" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="H72" s="6" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="I72" s="6"/>
       <c r="J72" s="5">
@@ -6047,13 +6047,13 @@
         <v>26</v>
       </c>
       <c r="N72" s="6" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="O72" s="6" t="s">
         <v>188</v>
       </c>
       <c r="P72" s="6" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="Q72" s="5">
         <v>46231</v>
@@ -6073,7 +6073,7 @@
     </row>
     <row r="73" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A73" s="7" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B73" s="8">
         <v>46111.50359008102</v>
@@ -6085,7 +6085,7 @@
         <v>46260.58097469907</v>
       </c>
       <c r="E73" s="9" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="F73" s="9" t="s">
         <v>25</v>
@@ -6109,7 +6109,7 @@
         <v>26</v>
       </c>
       <c r="O73" s="9" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="P73" s="9" t="s">
         <v>26</v>
@@ -6126,7 +6126,7 @@
     </row>
     <row r="74" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A74" s="4" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B74" s="5">
         <v>46111.50404616898</v>
@@ -6138,16 +6138,16 @@
         <v>46260.58079141204</v>
       </c>
       <c r="E74" s="6" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="F74" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G74" s="6" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="H74" s="6" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="I74" s="5">
         <v>46211</v>
@@ -6165,13 +6165,13 @@
         <v>26</v>
       </c>
       <c r="N74" s="6" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="O74" s="6" t="s">
         <v>169</v>
       </c>
       <c r="P74" s="6" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="Q74" s="5">
         <v>46211</v>
@@ -6191,7 +6191,7 @@
     </row>
     <row r="75" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A75" s="7" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B75" s="8">
         <v>46111.50406170139</v>
@@ -6203,16 +6203,16 @@
         <v>46260.580961342595</v>
       </c>
       <c r="E75" s="9" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="F75" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G75" s="9" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="H75" s="9" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="I75" s="8">
         <v>46213</v>
@@ -6230,13 +6230,13 @@
         <v>26</v>
       </c>
       <c r="N75" s="9" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="O75" s="9" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="P75" s="9" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="Q75" s="8">
         <v>46213</v>
@@ -6256,7 +6256,7 @@
     </row>
     <row r="76" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A76" s="4" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B76" s="5">
         <v>46111.50543856481</v>
@@ -6266,7 +6266,7 @@
         <v>46260.577887962965</v>
       </c>
       <c r="E76" s="6" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="F76" s="6" t="s">
         <v>25</v>
@@ -6290,7 +6290,7 @@
         <v>26</v>
       </c>
       <c r="O76" s="6" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="P76" s="6" t="s">
         <v>26</v>
@@ -6305,7 +6305,7 @@
     </row>
     <row r="77" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A77" s="7" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B77" s="8">
         <v>46111.505495046295</v>
@@ -6317,16 +6317,16 @@
         <v>46260.58096115741</v>
       </c>
       <c r="E77" s="9" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="F77" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G77" s="9" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="H77" s="9" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="I77" s="8">
         <v>46217</v>
@@ -6344,13 +6344,13 @@
         <v>26</v>
       </c>
       <c r="N77" s="9" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="O77" s="9" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="P77" s="9" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="Q77" s="8">
         <v>46217</v>
@@ -6370,7 +6370,7 @@
     </row>
     <row r="78" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A78" s="4" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B78" s="5">
         <v>46111.50560314815</v>
@@ -6382,16 +6382,16 @@
         <v>46260.57750302083</v>
       </c>
       <c r="E78" s="6" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="F78" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G78" s="6" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="H78" s="6" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="I78" s="5">
         <v>46226</v>
@@ -6409,13 +6409,13 @@
         <v>26</v>
       </c>
       <c r="N78" s="6" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="O78" s="6" t="s">
         <v>219</v>
       </c>
       <c r="P78" s="6" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="Q78" s="5">
         <v>46226</v>
@@ -6435,7 +6435,7 @@
     </row>
     <row r="79" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A79" s="7" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B79" s="8">
         <v>46111.52633317129</v>
@@ -6453,10 +6453,10 @@
         <v>26</v>
       </c>
       <c r="G79" s="9" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="H79" s="9" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="I79" s="8">
         <v>46226</v>
@@ -6474,13 +6474,13 @@
         <v>26</v>
       </c>
       <c r="N79" s="9" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="O79" s="9" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="P79" s="9" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="Q79" s="9"/>
       <c r="R79" s="9"/>
@@ -6490,7 +6490,7 @@
     </row>
     <row r="80" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A80" s="4" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B80" s="5">
         <v>46111.526644375</v>
@@ -6508,10 +6508,10 @@
         <v>26</v>
       </c>
       <c r="G80" s="6" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="H80" s="6" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="I80" s="5">
         <v>46226</v>
@@ -6529,13 +6529,13 @@
         <v>26</v>
       </c>
       <c r="N80" s="6" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="O80" s="6" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="P80" s="6" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="Q80" s="6"/>
       <c r="R80" s="6"/>
@@ -6545,7 +6545,7 @@
     </row>
     <row r="81" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A81" s="7" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B81" s="8">
         <v>46111.50563458333</v>
@@ -6557,16 +6557,16 @@
         <v>46260.57788128473</v>
       </c>
       <c r="E81" s="9" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="F81" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G81" s="9" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="H81" s="9" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="I81" s="8">
         <v>46246</v>
@@ -6584,13 +6584,13 @@
         <v>26</v>
       </c>
       <c r="N81" s="9" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="O81" s="9" t="s">
         <v>219</v>
       </c>
       <c r="P81" s="9" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="Q81" s="8">
         <v>46246</v>
@@ -6610,7 +6610,7 @@
     </row>
     <row r="82" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A82" s="4" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B82" s="5">
         <v>46111.526916469906</v>
@@ -6628,10 +6628,10 @@
         <v>26</v>
       </c>
       <c r="G82" s="6" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="H82" s="6" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="I82" s="5">
         <v>46246</v>
@@ -6649,13 +6649,13 @@
         <v>26</v>
       </c>
       <c r="N82" s="6" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="O82" s="6" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="P82" s="6" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="Q82" s="6"/>
       <c r="R82" s="6"/>
@@ -6665,7 +6665,7 @@
     </row>
     <row r="83" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A83" s="7" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B83" s="8">
         <v>46111.52699828704</v>
@@ -6683,10 +6683,10 @@
         <v>26</v>
       </c>
       <c r="G83" s="9" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="H83" s="9" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="I83" s="8">
         <v>46246</v>
@@ -6704,13 +6704,13 @@
         <v>26</v>
       </c>
       <c r="N83" s="9" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="O83" s="9" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="P83" s="9" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="Q83" s="9"/>
       <c r="R83" s="9"/>
@@ -6720,7 +6720,7 @@
     </row>
     <row r="84" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A84" s="4" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B84" s="5">
         <v>46108.75714884259</v>
@@ -6730,7 +6730,7 @@
         <v>46221.1155655787</v>
       </c>
       <c r="E84" s="6" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="F84" s="6" t="s">
         <v>25</v>
@@ -6754,7 +6754,7 @@
         <v>26</v>
       </c>
       <c r="O84" s="6" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="P84" s="6" t="s">
         <v>26</v>
@@ -6767,7 +6767,7 @@
     </row>
     <row r="85" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A85" s="7" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B85" s="8">
         <v>46108.75715243055</v>
@@ -6777,16 +6777,16 @@
         <v>46185.184959907405</v>
       </c>
       <c r="E85" s="9" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="F85" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G85" s="9" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="H85" s="9" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="I85" s="8">
         <v>46183</v>
@@ -6804,13 +6804,13 @@
         <v>26</v>
       </c>
       <c r="N85" s="9" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="O85" s="9" t="s">
         <v>147</v>
       </c>
       <c r="P85" s="9" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="Q85" s="8">
         <v>46183</v>
@@ -6830,7 +6830,7 @@
     </row>
     <row r="86" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A86" s="4" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="B86" s="5">
         <v>46108.75715773148</v>
@@ -6846,10 +6846,10 @@
         <v>26</v>
       </c>
       <c r="G86" s="6" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="H86" s="6" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="I86" s="5">
         <v>46239</v>
@@ -6867,13 +6867,13 @@
         <v>26</v>
       </c>
       <c r="N86" s="6" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="O86" s="6" t="s">
         <v>138</v>
       </c>
       <c r="P86" s="6" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="Q86" s="5">
         <v>46239</v>
@@ -6893,7 +6893,7 @@
     </row>
     <row r="87" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A87" s="7" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B87" s="8">
         <v>46108.75716349537</v>
@@ -6903,16 +6903,16 @@
         <v>46248.16971915509</v>
       </c>
       <c r="E87" s="9" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="F87" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G87" s="9" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="H87" s="9" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="I87" s="8">
         <v>46246</v>
@@ -6930,13 +6930,13 @@
         <v>26</v>
       </c>
       <c r="N87" s="9" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="O87" s="9" t="s">
         <v>129</v>
       </c>
       <c r="P87" s="9" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="Q87" s="8">
         <v>46246</v>
@@ -6956,26 +6956,26 @@
     </row>
     <row r="88" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A88" s="4" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="B88" s="5">
         <v>46108.75716875</v>
       </c>
       <c r="C88" s="6"/>
       <c r="D88" s="5">
-        <v>46267.17843465278</v>
+        <v>46274.167405914355</v>
       </c>
       <c r="E88" s="6" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="F88" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G88" s="6" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="H88" s="6" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="I88" s="5">
         <v>46273</v>
@@ -6993,13 +6993,13 @@
         <v>26</v>
       </c>
       <c r="N88" s="6" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="O88" s="6" t="s">
         <v>156</v>
       </c>
       <c r="P88" s="6" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="Q88" s="5">
         <v>46273</v>
@@ -7011,7 +7011,7 @@
         <v>0</v>
       </c>
       <c r="T88" s="12" t="s">
-        <v>298</v>
+        <v>238</v>
       </c>
       <c r="U88" s="10" t="s">
         <v>53</v>
@@ -7035,10 +7035,10 @@
         <v>26</v>
       </c>
       <c r="G89" s="9" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="H89" s="9" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="I89" s="8">
         <v>46220</v>
@@ -7056,7 +7056,7 @@
         <v>26</v>
       </c>
       <c r="N89" s="9" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="O89" s="9" t="s">
         <v>178</v>
@@ -7098,10 +7098,10 @@
         <v>26</v>
       </c>
       <c r="G90" s="6" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="H90" s="6" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="I90" s="6"/>
       <c r="J90" s="5">
@@ -7117,10 +7117,10 @@
         <v>26</v>
       </c>
       <c r="N90" s="6" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="O90" s="6" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="P90" s="6" t="s">
         <v>303</v>
@@ -7159,10 +7159,10 @@
         <v>26</v>
       </c>
       <c r="G91" s="9" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="H91" s="9" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="I91" s="8">
         <v>46181</v>
@@ -7180,7 +7180,7 @@
         <v>26</v>
       </c>
       <c r="N91" s="9" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="O91" s="9" t="s">
         <v>198</v>
@@ -7598,7 +7598,7 @@
       </c>
       <c r="C99" s="9"/>
       <c r="D99" s="8">
-        <v>46273.16745574074</v>
+        <v>46274.149059386575</v>
       </c>
       <c r="E99" s="9" t="s">
         <v>327</v>
@@ -7645,8 +7645,8 @@
       <c r="S99" s="9">
         <v>0</v>
       </c>
-      <c r="T99" s="12" t="s">
-        <v>298</v>
+      <c r="T99" s="10" t="s">
+        <v>31</v>
       </c>
       <c r="U99" s="10" t="s">
         <v>53</v>
@@ -7815,7 +7815,7 @@
         <v>0</v>
       </c>
       <c r="T102" s="12" t="s">
-        <v>298</v>
+        <v>238</v>
       </c>
       <c r="U102" s="10" t="s">
         <v>53</v>
@@ -7984,7 +7984,7 @@
         <v>0</v>
       </c>
       <c r="T105" s="12" t="s">
-        <v>298</v>
+        <v>238</v>
       </c>
       <c r="U105" s="10" t="s">
         <v>53</v>
@@ -8153,7 +8153,7 @@
         <v>0</v>
       </c>
       <c r="T108" s="12" t="s">
-        <v>298</v>
+        <v>238</v>
       </c>
       <c r="U108" s="10" t="s">
         <v>53</v>
@@ -8413,7 +8413,7 @@
         <v>355</v>
       </c>
       <c r="O113" s="9" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="P113" s="9" t="s">
         <v>360</v>
@@ -9343,10 +9343,10 @@
         <v>26</v>
       </c>
       <c r="G131" s="9" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="H131" s="9" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="I131" s="8">
         <v>46293</v>
@@ -9406,10 +9406,10 @@
         <v>26</v>
       </c>
       <c r="G132" s="6" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="H132" s="6" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="I132" s="6"/>
       <c r="J132" s="5">
@@ -9457,10 +9457,10 @@
         <v>26</v>
       </c>
       <c r="G133" s="9" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="H133" s="9" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="I133" s="9"/>
       <c r="J133" s="8">
@@ -9508,10 +9508,10 @@
         <v>26</v>
       </c>
       <c r="G134" s="6" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="H134" s="6" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="I134" s="6"/>
       <c r="J134" s="5">
@@ -9559,10 +9559,10 @@
         <v>26</v>
       </c>
       <c r="G135" s="9" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="H135" s="9" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="I135" s="9"/>
       <c r="J135" s="8">
@@ -9610,10 +9610,10 @@
         <v>26</v>
       </c>
       <c r="G136" s="6" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="H136" s="6" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="I136" s="6"/>
       <c r="J136" s="5">
@@ -9661,10 +9661,10 @@
         <v>26</v>
       </c>
       <c r="G137" s="9" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="H137" s="9" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="I137" s="9"/>
       <c r="J137" s="8">
@@ -9712,10 +9712,10 @@
         <v>26</v>
       </c>
       <c r="G138" s="6" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="H138" s="6" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="I138" s="6"/>
       <c r="J138" s="5">
@@ -9763,10 +9763,10 @@
         <v>26</v>
       </c>
       <c r="G139" s="9" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="H139" s="9" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="I139" s="8">
         <v>46294</v>
@@ -9826,10 +9826,10 @@
         <v>26</v>
       </c>
       <c r="G140" s="6" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="H140" s="6" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="I140" s="5">
         <v>46294</v>
@@ -9879,10 +9879,10 @@
         <v>26</v>
       </c>
       <c r="G141" s="9" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="H141" s="9" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="I141" s="8">
         <v>46294</v>
@@ -9932,10 +9932,10 @@
         <v>26</v>
       </c>
       <c r="G142" s="6" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="H142" s="6" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="I142" s="5">
         <v>46294</v>
@@ -9985,10 +9985,10 @@
         <v>26</v>
       </c>
       <c r="G143" s="9" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="H143" s="9" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="I143" s="8">
         <v>46294</v>
@@ -10038,10 +10038,10 @@
         <v>26</v>
       </c>
       <c r="G144" s="6" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="H144" s="6" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="I144" s="5">
         <v>46294</v>
@@ -10091,10 +10091,10 @@
         <v>26</v>
       </c>
       <c r="G145" s="9" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="H145" s="9" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="I145" s="8">
         <v>46294</v>
@@ -10144,10 +10144,10 @@
         <v>26</v>
       </c>
       <c r="G146" s="6" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="H146" s="6" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="I146" s="5">
         <v>46294</v>

</xml_diff>

<commit_message>
Actualiza portafolio 2026-09-11 17:09 UTC
</commit_message>
<xml_diff>
--- a/data/50001525 - ZITRON PERU METRO LIMA E07.xlsx
+++ b/data/50001525 - ZITRON PERU METRO LIMA E07.xlsx
@@ -7767,7 +7767,7 @@
       </c>
       <c r="C102" s="6"/>
       <c r="D102" s="5">
-        <v>46275.16746550926</v>
+        <v>46276.143129421296</v>
       </c>
       <c r="E102" s="6" t="s">
         <v>335</v>
@@ -7814,8 +7814,8 @@
       <c r="S102" s="6">
         <v>0</v>
       </c>
-      <c r="T102" s="12" t="s">
-        <v>238</v>
+      <c r="T102" s="10" t="s">
+        <v>31</v>
       </c>
       <c r="U102" s="10" t="s">
         <v>53</v>

</xml_diff>